<commit_message>
Update FIRIS forecast 2026-09-20
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'مناطق_چهارگانه'!$A$1:$H$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'مناطق_شکار_ممنوع'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'طبقات_خطر'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'طبقات_خطر'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,14 +48,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="B Nazanin"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,17 +68,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDD835"/>
+        <fgColor rgb="00E53935"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E53935"/>
+        <fgColor rgb="00C7A900"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -130,19 +119,16 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -545,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-10.tif</t>
+          <t>fli_fars_2026-09-20.tif</t>
         </is>
       </c>
     </row>
@@ -568,7 +554,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>904753</v>
+        <v>1783231</v>
       </c>
     </row>
     <row r="7">
@@ -588,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>71.45</v>
+        <v>87.68000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>42.66</v>
+        <v>36.11</v>
       </c>
     </row>
     <row r="10">
@@ -620,7 +606,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.002588441050000003</v>
+        <v>0.002589577909999999</v>
       </c>
     </row>
     <row r="12">
@@ -630,7 +616,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.002411990949999999</v>
+        <v>0.002410847090000002</v>
       </c>
     </row>
   </sheetData>
@@ -718,20 +704,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>40.85</v>
+        <v>52.76</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.62</v>
+        <v>26.91</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>58.4</v>
+        <v>80.03</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>24441</v>
+        <v>24931</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -750,20 +736,20 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>47.22</v>
+        <v>51</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>32.28</v>
+        <v>29.89</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>63.75</v>
+        <v>83</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>5703</v>
+        <v>7596</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -782,16 +768,16 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>24.85</v>
+        <v>19.67</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>42.9</v>
+        <v>70.77</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>751</v>
+        <v>14316</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
@@ -814,18 +800,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>50.87</v>
+        <v>42.76</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>41.52</v>
+        <v>27.34</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>64.38</v>
+        <v>67.22</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>10563</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+        <v>13047</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -846,18 +832,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>43.14</v>
+        <v>41.52</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>36.75</v>
+        <v>25.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>53.41</v>
+        <v>61.6</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>1663</v>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+        <v>4435</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -878,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>56.71</v>
+        <v>50.37</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>49.26</v>
+        <v>29.47</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>68.58</v>
+        <v>70.25</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>2137</v>
+        <v>2330</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -910,18 +896,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>43.13</v>
+        <v>32.88</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>1.01</v>
+        <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>65.12</v>
+        <v>56.08</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>1950</v>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+        <v>4168</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -942,20 +928,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>33.48</v>
+        <v>45.62</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>26.69</v>
+        <v>32.93</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>45.11</v>
+        <v>65.59</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>187</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>1294</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -974,18 +960,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>49.39</v>
+        <v>27.98</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>40.25</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>61.49</v>
+        <v>59.77</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>1059</v>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+        <v>3417</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1006,18 +992,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>41.68</v>
+        <v>46.21</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.97</v>
+        <v>28.13</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.65</v>
+        <v>68.81</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>3976</v>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+        <v>4643</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1038,18 +1024,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.78</v>
+        <v>48.18</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>35.79</v>
+        <v>27.59</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>57.86</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>5465</v>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+        <v>8020</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1070,18 +1056,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>49.48</v>
+        <v>45.81</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>33.34</v>
+        <v>27.46</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>68.90000000000001</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>6849</v>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+        <v>13859</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1102,16 +1088,16 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>24.93</v>
+        <v>23.81</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>1.06</v>
+        <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>35.13</v>
+        <v>58.44</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>79</v>
+        <v>10541</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -1134,16 +1120,16 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>31.66</v>
+        <v>23.92</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0.45</v>
+        <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>53.66</v>
+        <v>58.24</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>932</v>
+        <v>13329</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
@@ -1166,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>47.18</v>
+        <v>53.89</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>35.37</v>
+        <v>28.61</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>62.68</v>
+        <v>76.95</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>4808</v>
+        <v>4909</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1198,20 +1184,20 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>33.13</v>
+        <v>28.89</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>1.32</v>
+        <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.18</v>
+        <v>56.66</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>4944</v>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>19003</v>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1230,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>31.73</v>
+        <v>40.11</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0.65</v>
+        <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>48.2</v>
+        <v>68.48</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>5180</v>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>11473</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1262,18 +1248,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>44.92</v>
+        <v>38.47</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>0.59</v>
+        <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>62.1</v>
+        <v>65.09</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>3925</v>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+        <v>9100</v>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1294,18 +1280,18 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>48.47</v>
+        <v>47.94</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>37.99</v>
+        <v>30.18</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>58.64</v>
+        <v>66.66</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>657</v>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+        <v>791</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1326,18 +1312,18 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46.11</v>
+        <v>49.09</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>30.35</v>
+        <v>29.63</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>63.11</v>
+        <v>69.42</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>6257</v>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+        <v>7038</v>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1358,20 +1344,20 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>17.14</v>
+        <v>15.7</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>3.47</v>
+        <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>36.24</v>
+        <v>50.53</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>کم</t>
+        <v>4821</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1458,20 +1444,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>38.67</v>
+        <v>48.84</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.98</v>
+        <v>29.94</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>51.44</v>
+        <v>71.56</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>2293</v>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>2287</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1490,18 +1476,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>49.65</v>
+        <v>44.81</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>40.32</v>
+        <v>24.87</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.70999999999999</v>
+        <v>71.31</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>4823</v>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
+        <v>7892</v>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1522,16 +1508,16 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>25.86</v>
+        <v>16.73</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.55</v>
+        <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>49.9</v>
+        <v>66.19</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>868</v>
+        <v>18742</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
@@ -1554,18 +1540,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>48.84</v>
+        <v>47.94</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>37.96</v>
+        <v>33.72</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>61.01</v>
+        <v>61.23</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>466</v>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+        <v>470</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1586,16 +1572,16 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>32.75</v>
+        <v>9.4</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>64.09</v>
+        <v>56.99</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>2048</v>
+        <v>43913</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -1618,20 +1604,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>44.55</v>
+        <v>11.52</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>6.54</v>
+        <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>53.6</v>
+        <v>51.04</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>173</v>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+        <v>4718</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1650,18 +1636,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>45.4</v>
+        <v>48</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>35.48</v>
+        <v>28.4</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>62.12</v>
+        <v>73.38</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>7042</v>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+        <v>8411</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1682,16 +1668,16 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>21.55</v>
+        <v>19.16</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>9.050000000000001</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>42.9</v>
+        <v>53.58</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>66</v>
+        <v>2525</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
@@ -1714,18 +1700,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.44</v>
+        <v>48.48</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>37.12</v>
+        <v>28.01</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>60.09</v>
+        <v>74.05</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>6931</v>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+        <v>7186</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1746,18 +1732,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>52.09</v>
+        <v>45.5</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>39.99</v>
+        <v>27.18</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.69</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>5654</v>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+        <v>6990</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1778,18 +1764,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>48.46</v>
+        <v>34</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>65.34</v>
+        <v>77.76000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>16529</v>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+        <v>45935</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1810,18 +1796,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>48.33</v>
+        <v>28.72</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>4.03</v>
+        <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>65.34</v>
+        <v>58.8</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>5265</v>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+        <v>24115</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1842,18 +1828,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>44.01</v>
+        <v>48.82</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>34.33</v>
+        <v>29.92</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>55.59</v>
+        <v>66.95999999999999</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>2311</v>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+        <v>2712</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1874,18 +1860,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>57.33</v>
+        <v>47.25</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>49.35</v>
+        <v>32.06</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>70.2</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>1185</v>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+        <v>1692</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1904,7 +1890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1942,102 +1928,83 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>کم</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39049</v>
+        <v>298063</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>4.32</v>
+        <v>16.71</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>235620</v>
+        <v>1218277</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>26.04</v>
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>خیلی زیاد</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>621456</v>
+        <v>266447</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>68.69</v>
+        <v>14.94</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>بحرانی</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>8628</v>
+        <v>444</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>بحرانی</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>80</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:E5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2095,7 +2062,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0.002588441050000003</v>
+        <v>0.002589577909999999</v>
       </c>
     </row>
     <row r="5">
@@ -2105,7 +2072,7 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.002411990949999999</v>
+        <v>0.002410847090000002</v>
       </c>
     </row>
     <row r="6">
@@ -2115,7 +2082,7 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>50.5031831</v>
+        <v>50.50271989</v>
       </c>
     </row>
     <row r="7">
@@ -2125,7 +2092,7 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>26.945617</v>
+        <v>26.95024464999999</v>
       </c>
     </row>
     <row r="8">
@@ -2135,7 +2102,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>55.68006520000001</v>
+        <v>55.68187571</v>
       </c>
     </row>
     <row r="9">
@@ -2145,7 +2112,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>31.7695989</v>
+        <v>31.77193883</v>
       </c>
     </row>
     <row r="10">
@@ -2155,7 +2122,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.002588441050000003</v>
+        <v>0.002589577909999999</v>
       </c>
     </row>
     <row r="11">
@@ -2175,7 +2142,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>50.5031831</v>
+        <v>50.50271989</v>
       </c>
     </row>
     <row r="13">
@@ -2195,7 +2162,7 @@
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>-0.002411990949999999</v>
+        <v>-0.002410847090000002</v>
       </c>
     </row>
     <row r="15">
@@ -2205,7 +2172,7 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>31.7695989</v>
+        <v>31.77193883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-21
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -122,10 +122,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-20.tif</t>
+          <t>fli_fars_2026-09-21.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>87.68000000000001</v>
+        <v>93.19</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>36.11</v>
+        <v>36.81</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52.76</v>
+        <v>53.81</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.91</v>
+        <v>28.62</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>80.03</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,20 +736,20 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>51</v>
+        <v>49.9</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.89</v>
+        <v>28.75</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>83</v>
+        <v>80.62</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -768,18 +768,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>19.67</v>
+        <v>17.94</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>70.77</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -800,18 +800,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>42.76</v>
+        <v>49.22</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.34</v>
+        <v>30.09</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>67.22</v>
+        <v>73.58</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -832,18 +832,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>41.52</v>
+        <v>45.08</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>25.21</v>
+        <v>27.81</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>61.6</v>
+        <v>66.77</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.37</v>
+        <v>53.54</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>29.47</v>
+        <v>32.83</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>70.25</v>
+        <v>74.62</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,18 +896,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>32.88</v>
+        <v>33.08</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>56.08</v>
+        <v>55.75</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -928,18 +928,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>45.62</v>
+        <v>38.55</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>32.93</v>
+        <v>27.32</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>65.59</v>
+        <v>56.94</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -960,18 +960,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>27.98</v>
+        <v>30.01</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>59.77</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -992,18 +992,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46.21</v>
+        <v>49.26</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.13</v>
+        <v>32.34</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.81</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1024,18 +1024,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>48.18</v>
+        <v>47.75</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>27.59</v>
+        <v>27.64</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>77.09999999999999</v>
+        <v>76.34</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1056,18 +1056,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>45.81</v>
+        <v>44.92</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>27.46</v>
+        <v>26.35</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>69.84999999999999</v>
+        <v>71.31</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1088,18 +1088,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.81</v>
+        <v>22.71</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>58.44</v>
+        <v>52.94</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1120,18 +1120,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.92</v>
+        <v>23.3</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.24</v>
+        <v>57.89</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>53.89</v>
+        <v>57.15</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>28.61</v>
+        <v>31.68</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>76.95</v>
+        <v>79.55</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,18 +1184,18 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.89</v>
+        <v>29.14</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.66</v>
+        <v>56.93</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1216,18 +1216,18 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>40.11</v>
+        <v>39.83</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>68.48</v>
+        <v>65.56</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1248,18 +1248,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>38.47</v>
+        <v>38.36</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>65.09</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47.94</v>
+        <v>52.77</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>30.18</v>
+        <v>35.18</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.66</v>
+        <v>70.54000000000001</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,20 +1312,20 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>49.09</v>
+        <v>50.63</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>29.63</v>
+        <v>32.17</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>69.42</v>
+        <v>70.95</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1344,18 +1344,18 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>15.7</v>
+        <v>15.75</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>50.53</v>
+        <v>50.27</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1444,18 +1444,18 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.84</v>
+        <v>49.15</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>29.94</v>
+        <v>26.65</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>71.56</v>
+        <v>69.88</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1476,18 +1476,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.81</v>
+        <v>46.24</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>24.87</v>
+        <v>30.33</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>71.31</v>
+        <v>71.86</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1508,18 +1508,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.73</v>
+        <v>15.2</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>66.19</v>
+        <v>56.45</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>47.94</v>
+        <v>54.95</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>33.72</v>
+        <v>36.77</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>61.23</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,18 +1572,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.4</v>
+        <v>9.74</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>56.99</v>
+        <v>58.06</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1604,18 +1604,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.52</v>
+        <v>10.91</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>51.04</v>
+        <v>47.95</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1636,20 +1636,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>48</v>
+        <v>50.68</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>28.4</v>
+        <v>31.32</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>73.38</v>
+        <v>76.43000000000001</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1668,18 +1668,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>19.16</v>
+        <v>17.91</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>53.58</v>
+        <v>50.81</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1700,18 +1700,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>48.48</v>
+        <v>49.66</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>28.01</v>
+        <v>29.86</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>74.05</v>
+        <v>73.69</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1732,18 +1732,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.5</v>
+        <v>47.31</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.18</v>
+        <v>27.83</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>65.40000000000001</v>
+        <v>69.61</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1764,18 +1764,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>34</v>
+        <v>34.45</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>77.76000000000001</v>
+        <v>79.41</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1796,18 +1796,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>28.72</v>
+        <v>29.54</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>58.8</v>
+        <v>61.99</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>48.82</v>
+        <v>52.33</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>29.92</v>
+        <v>35.2</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>66.95999999999999</v>
+        <v>70.75</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1860,18 +1860,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>47.25</v>
+        <v>49.4</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>32.06</v>
+        <v>34.9</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>64.76000000000001</v>
+        <v>64.08</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1928,7 +1928,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1940,14 +1940,14 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>298063</v>
+        <v>303786</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>16.71</v>
+        <v>17.04</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1218277</v>
+        <v>1152019</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>68.31999999999999</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>266447</v>
+        <v>325947</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>14.94</v>
+        <v>18.28</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>444</v>
+        <v>1479</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-22
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-21.tif</t>
+          <t>fli_fars_2026-09-22.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>93.19</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>36.81</v>
+        <v>34.78</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>53.81</v>
+        <v>52.25</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.62</v>
+        <v>26.93</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>80.31999999999999</v>
+        <v>78.45</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>49.9</v>
+        <v>48.64</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.75</v>
+        <v>27.94</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>80.62</v>
+        <v>79.95999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>17.94</v>
+        <v>19.12</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>64.51000000000001</v>
+        <v>71.45999999999999</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>49.22</v>
+        <v>48.33</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.09</v>
+        <v>30.35</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>73.58</v>
+        <v>73.37</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>45.08</v>
+        <v>42.96</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>27.81</v>
+        <v>28.18</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>66.77</v>
+        <v>62.89</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>53.54</v>
+        <v>51.13</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>32.83</v>
+        <v>28.5</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>74.62</v>
+        <v>69.58</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.08</v>
+        <v>34.63</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.75</v>
+        <v>58.44</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>38.55</v>
+        <v>43.39</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>27.32</v>
+        <v>31.59</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>56.94</v>
+        <v>64.45999999999999</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>30.01</v>
+        <v>27.96</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>64.56999999999999</v>
+        <v>60.73</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>49.26</v>
+        <v>46.21</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>32.34</v>
+        <v>29.15</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>70.48999999999999</v>
+        <v>68.55</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>47.75</v>
+        <v>45.37</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>27.64</v>
+        <v>25.38</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>76.34</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.92</v>
+        <v>43.3</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>26.35</v>
+        <v>26.06</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>71.31</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.71</v>
+        <v>23.3</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>52.94</v>
+        <v>56.72</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.3</v>
+        <v>23.77</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.89</v>
+        <v>59.7</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>57.15</v>
+        <v>52.88</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>31.68</v>
+        <v>26.94</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>79.55</v>
+        <v>75.48</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>29.14</v>
+        <v>26.57</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.93</v>
+        <v>53</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>39.83</v>
+        <v>38.35</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>65.56</v>
+        <v>62.47</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>38.36</v>
+        <v>35.27</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>65.26000000000001</v>
+        <v>60.81</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>52.77</v>
+        <v>49.64</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>35.18</v>
+        <v>29.67</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>70.54000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,20 +1312,20 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>50.63</v>
+        <v>47.02</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>32.17</v>
+        <v>29.02</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>70.95</v>
+        <v>67.23999999999999</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>15.75</v>
+        <v>14.61</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>50.27</v>
+        <v>45.89</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>49.15</v>
+        <v>49.1</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.65</v>
+        <v>31.39</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>69.88</v>
+        <v>71.98</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46.24</v>
+        <v>45.92</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>30.33</v>
+        <v>29.07</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>71.86</v>
+        <v>70.86</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.2</v>
+        <v>14.8</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>56.45</v>
+        <v>57.85</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>54.95</v>
+        <v>43.04</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>36.77</v>
+        <v>27.02</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.73999999999999</v>
+        <v>54.23</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.74</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>58.06</v>
+        <v>54.1</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.91</v>
+        <v>10.65</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>47.95</v>
+        <v>48.34</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,20 +1636,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>50.68</v>
+        <v>46.6</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>31.32</v>
+        <v>27.02</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>76.43000000000001</v>
+        <v>73.73999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>17.91</v>
+        <v>19.21</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>50.81</v>
+        <v>51.74</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>49.66</v>
+        <v>46.8</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>29.86</v>
+        <v>26.67</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>73.69</v>
+        <v>72.39</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>47.31</v>
+        <v>47.38</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.83</v>
+        <v>27.32</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>69.61</v>
+        <v>68.59</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>34.45</v>
+        <v>32.87</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>79.41</v>
+        <v>75.47</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>29.54</v>
+        <v>27.73</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>61.99</v>
+        <v>56.71</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>52.33</v>
+        <v>46.66</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>35.2</v>
+        <v>28.02</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>70.75</v>
+        <v>63.6</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>49.4</v>
+        <v>50.72</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>34.9</v>
+        <v>36.52</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>64.08</v>
+        <v>67.19</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>303786</v>
+        <v>329064</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.04</v>
+        <v>18.45</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1152019</v>
+        <v>1229196</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>64.59999999999999</v>
+        <v>68.93000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>325947</v>
+        <v>224478</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>18.28</v>
+        <v>12.59</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>1479</v>
+        <v>493</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-24
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-22.tif</t>
+          <t>fli_fars_2026-09-24.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>90.90000000000001</v>
+        <v>91.8</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.78</v>
+        <v>35.23</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52.25</v>
+        <v>52</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.93</v>
+        <v>25.7</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>78.45</v>
+        <v>79.7</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>48.64</v>
+        <v>48.65</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>27.94</v>
+        <v>28.73</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>79.95999999999999</v>
+        <v>81.42</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>19.12</v>
+        <v>19.93</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>71.45999999999999</v>
+        <v>73.62</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>48.33</v>
+        <v>46.45</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.35</v>
+        <v>30.46</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>73.37</v>
+        <v>70.97</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>42.96</v>
+        <v>44.32</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>28.18</v>
+        <v>28.91</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>62.89</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.13</v>
+        <v>51.21</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>28.5</v>
+        <v>30.25</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>69.58</v>
+        <v>71.02</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.63</v>
+        <v>33.03</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>58.44</v>
+        <v>55.36</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>43.39</v>
+        <v>46.69</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>31.59</v>
+        <v>35.87</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>64.45999999999999</v>
+        <v>69.02</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>27.96</v>
+        <v>27.99</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>60.73</v>
+        <v>58.26</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46.21</v>
+        <v>44.61</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>29.15</v>
+        <v>25.59</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.55</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.37</v>
+        <v>45.23</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.38</v>
+        <v>25.83</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.01000000000001</v>
+        <v>73.12</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>43.3</v>
+        <v>44.73</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>26.06</v>
+        <v>27.04</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>66.56999999999999</v>
+        <v>69.02</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.3</v>
+        <v>22.34</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>56.72</v>
+        <v>54.34</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.77</v>
+        <v>22.91</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>59.7</v>
+        <v>56.56</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.88</v>
+        <v>52.96</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>26.94</v>
+        <v>25.48</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.48</v>
+        <v>75.15000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.57</v>
+        <v>27.6</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53</v>
+        <v>55.14</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>38.35</v>
+        <v>41.25</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>62.47</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>35.27</v>
+        <v>36.42</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>60.81</v>
+        <v>62.88</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>49.64</v>
+        <v>51.14</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>29.67</v>
+        <v>32.53</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>68.7</v>
+        <v>70.63</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>47.02</v>
+        <v>46.57</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>29.02</v>
+        <v>25.14</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>67.23999999999999</v>
+        <v>71.42</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14.61</v>
+        <v>14.57</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>45.89</v>
+        <v>45.08</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>49.1</v>
+        <v>48.85</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>31.39</v>
+        <v>31.87</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>71.98</v>
+        <v>71.23</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45.92</v>
+        <v>44.77</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.07</v>
+        <v>29.06</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>70.86</v>
+        <v>70.23</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.8</v>
+        <v>15.86</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>57.85</v>
+        <v>65.11</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>43.04</v>
+        <v>51.47</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.02</v>
+        <v>32.36</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>54.23</v>
+        <v>63.66</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.210000000000001</v>
+        <v>9.91</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.1</v>
+        <v>57.1</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.65</v>
+        <v>12.04</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>48.34</v>
+        <v>52.72</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46.6</v>
+        <v>47.67</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>27.02</v>
+        <v>26.69</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>73.73999999999999</v>
+        <v>74.76000000000001</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>19.21</v>
+        <v>19.91</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>51.74</v>
+        <v>53.52</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.8</v>
+        <v>46.06</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>26.67</v>
+        <v>26.4</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>72.39</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>47.38</v>
+        <v>45.6</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.32</v>
+        <v>26.54</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.59</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.87</v>
+        <v>34.85</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>75.47</v>
+        <v>78.27</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>27.73</v>
+        <v>29.17</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>56.71</v>
+        <v>61.41</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46.66</v>
+        <v>47.05</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>28.02</v>
+        <v>27.74</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>63.6</v>
+        <v>64.09</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>50.72</v>
+        <v>48.16</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>36.52</v>
+        <v>33.22</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>67.19</v>
+        <v>65.02</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>329064</v>
+        <v>316732</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.45</v>
+        <v>17.76</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1229196</v>
+        <v>1235201</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>68.93000000000001</v>
+        <v>69.27</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>224478</v>
+        <v>230489</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>12.59</v>
+        <v>12.93</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>493</v>
+        <v>809</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-25
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-24.tif</t>
+          <t>fli_fars_2026-09-25.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>91.8</v>
+        <v>89.8</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>35.23</v>
+        <v>35.69</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52</v>
+        <v>53.02</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.7</v>
+        <v>26.27</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>79.7</v>
+        <v>79.87</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>48.65</v>
+        <v>48.98</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.73</v>
+        <v>29.69</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>81.42</v>
+        <v>81.89</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>19.93</v>
+        <v>20.67</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>73.62</v>
+        <v>76.42</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46.45</v>
+        <v>45.75</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.46</v>
+        <v>29.75</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>70.97</v>
+        <v>70.69</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>44.32</v>
+        <v>43.65</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>28.91</v>
+        <v>28.09</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>64.20999999999999</v>
+        <v>64.11</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.21</v>
+        <v>50.61</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>30.25</v>
+        <v>29.21</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>71.02</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.03</v>
+        <v>37.43</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.36</v>
+        <v>62.2</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>46.69</v>
+        <v>47.23</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>35.87</v>
+        <v>35.38</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>69.02</v>
+        <v>69.91</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>27.99</v>
+        <v>28.33</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>58.26</v>
+        <v>59.92</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>44.61</v>
+        <v>45.09</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.59</v>
+        <v>26.96</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.90000000000001</v>
+        <v>67.76000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.23</v>
+        <v>46.36</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.83</v>
+        <v>27.21</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.12</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.73</v>
+        <v>46.93</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>27.04</v>
+        <v>28.58</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>69.02</v>
+        <v>74.23</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.34</v>
+        <v>23.42</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>54.34</v>
+        <v>53.71</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.91</v>
+        <v>23.43</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.56</v>
+        <v>57.13</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.96</v>
+        <v>52.46</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>25.48</v>
+        <v>27.84</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.15000000000001</v>
+        <v>75.18000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.6</v>
+        <v>27.37</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>55.14</v>
+        <v>55.05</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>41.25</v>
+        <v>42.15</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>67.65000000000001</v>
+        <v>67.75</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>36.42</v>
+        <v>34.91</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>62.88</v>
+        <v>61.64</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>51.14</v>
+        <v>52.75</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>32.53</v>
+        <v>34.05</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>70.63</v>
+        <v>72.06999999999999</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>46.57</v>
+        <v>47.32</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>25.14</v>
+        <v>26.51</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>71.42</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14.57</v>
+        <v>15.67</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>45.08</v>
+        <v>51.64</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,20 +1444,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.85</v>
+        <v>51.02</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>31.87</v>
+        <v>32.66</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>71.23</v>
+        <v>73.39</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.77</v>
+        <v>44.24</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.06</v>
+        <v>28.7</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>70.23</v>
+        <v>70.42</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.86</v>
+        <v>16.02</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>65.11</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>51.47</v>
+        <v>46.26</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.36</v>
+        <v>27.72</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>63.66</v>
+        <v>58.02</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.91</v>
+        <v>9.92</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>57.1</v>
+        <v>59.73</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>12.04</v>
+        <v>12.16</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>52.72</v>
+        <v>53.02</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>47.67</v>
+        <v>48.48</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>26.69</v>
+        <v>31.45</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>74.76000000000001</v>
+        <v>75.28</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>19.91</v>
+        <v>20.58</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>53.52</v>
+        <v>56.88</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.06</v>
+        <v>47.48</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>26.4</v>
+        <v>27.42</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>72.56999999999999</v>
+        <v>74.55</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.6</v>
+        <v>46.86</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.54</v>
+        <v>28.22</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>65.98999999999999</v>
+        <v>67.70999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>34.85</v>
+        <v>34.26</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>78.27</v>
+        <v>76.87</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>29.17</v>
+        <v>28.8</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>61.41</v>
+        <v>60.27</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>47.05</v>
+        <v>47.87</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>27.74</v>
+        <v>27.68</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>64.09</v>
+        <v>64.78</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>48.16</v>
+        <v>49.96</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>33.22</v>
+        <v>36.23</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>65.02</v>
+        <v>65.75</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>316732</v>
+        <v>309866</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.76</v>
+        <v>17.38</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1235201</v>
+        <v>1218253</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>69.27</v>
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>230489</v>
+        <v>254650</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>12.93</v>
+        <v>14.28</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>809</v>
+        <v>462</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-27
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-25.tif</t>
+          <t>fli_fars_2026-09-27.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>89.8</v>
+        <v>88.31999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>35.69</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>53.02</v>
+        <v>52.16</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.27</v>
+        <v>28.41</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>79.87</v>
+        <v>78.79000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>48.98</v>
+        <v>49.13</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.69</v>
+        <v>28.87</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>81.89</v>
+        <v>81.59</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>20.67</v>
+        <v>18.01</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>76.42</v>
+        <v>66.69</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>45.75</v>
+        <v>46.6</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>29.75</v>
+        <v>30.57</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>70.69</v>
+        <v>71.84</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>43.65</v>
+        <v>43.49</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>28.09</v>
+        <v>26.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>64.11</v>
+        <v>64.05</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.61</v>
+        <v>50.1</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>29.21</v>
+        <v>29.28</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>69.98999999999999</v>
+        <v>70.06</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>37.43</v>
+        <v>36.85</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>62.2</v>
+        <v>62.67</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>47.23</v>
+        <v>39.34</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>35.38</v>
+        <v>27.35</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>69.91</v>
+        <v>59.81</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>28.33</v>
+        <v>29.3</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>59.92</v>
+        <v>59.18</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.09</v>
+        <v>47.54</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.96</v>
+        <v>28.53</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.76000000000001</v>
+        <v>69.12</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46.36</v>
+        <v>47.77</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>27.21</v>
+        <v>27.42</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.29000000000001</v>
+        <v>76.81999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46.93</v>
+        <v>46.75</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>28.58</v>
+        <v>25.61</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>74.23</v>
+        <v>70.55</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.42</v>
+        <v>23.48</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>53.71</v>
+        <v>53.08</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.43</v>
+        <v>23.25</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.13</v>
+        <v>56.72</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.46</v>
+        <v>54.92</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>27.84</v>
+        <v>28.83</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.18000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.37</v>
+        <v>30.76</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>55.05</v>
+        <v>58.58</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>42.15</v>
+        <v>37.91</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>67.75</v>
+        <v>63.95</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>34.91</v>
+        <v>38.1</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>61.64</v>
+        <v>66</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>52.75</v>
+        <v>47.69</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>34.05</v>
+        <v>30.46</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>72.06999999999999</v>
+        <v>65.87</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>47.32</v>
+        <v>47.25</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.51</v>
+        <v>29.6</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>70.79000000000001</v>
+        <v>68.52</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>15.67</v>
+        <v>15.14</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>51.64</v>
+        <v>48.38</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,20 +1444,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>51.02</v>
+        <v>45.23</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>32.66</v>
+        <v>25.96</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>73.39</v>
+        <v>65.22</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.24</v>
+        <v>46.56</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.7</v>
+        <v>29.05</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>70.42</v>
+        <v>72.72</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.02</v>
+        <v>15.91</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>65.31999999999999</v>
+        <v>63.78</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46.26</v>
+        <v>52.32</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.72</v>
+        <v>38.35</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>58.02</v>
+        <v>64.17</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.92</v>
+        <v>9.51</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.73</v>
+        <v>54.94</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>12.16</v>
+        <v>11.61</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>53.02</v>
+        <v>52.13</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>48.48</v>
+        <v>49.7</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>31.45</v>
+        <v>30.63</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>75.28</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>20.58</v>
+        <v>17.64</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>56.88</v>
+        <v>48.18</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,20 +1700,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>47.48</v>
+        <v>51.32</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27.42</v>
+        <v>28.99</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>74.55</v>
+        <v>75.63</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46.86</v>
+        <v>45.16</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.22</v>
+        <v>27.1</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.70999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>34.26</v>
+        <v>34.17</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>76.87</v>
+        <v>79.39</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>28.8</v>
+        <v>29.23</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>60.27</v>
+        <v>62.13</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>47.87</v>
+        <v>49.38</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>27.68</v>
+        <v>33.12</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>64.78</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>49.96</v>
+        <v>47.71</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>36.23</v>
+        <v>33.09</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>65.75</v>
+        <v>62.27</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>309866</v>
+        <v>298407</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.38</v>
+        <v>16.73</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1218253</v>
+        <v>1192244</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>68.31999999999999</v>
+        <v>66.86</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>254650</v>
+        <v>291952</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>14.28</v>
+        <v>16.37</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>462</v>
+        <v>628</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-30
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-27.tif</t>
+          <t>fli_fars_2026-09-30.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>88.31999999999999</v>
+        <v>93.19</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>36.25</v>
+        <v>36.46</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52.16</v>
+        <v>52.13</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.41</v>
+        <v>26.95</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>78.79000000000001</v>
+        <v>78.31</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>49.13</v>
+        <v>46.74</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.87</v>
+        <v>26.66</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>81.59</v>
+        <v>79.23999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.01</v>
+        <v>18.58</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>66.69</v>
+        <v>69.39</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,20 +800,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46.6</v>
+        <v>50.08</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.57</v>
+        <v>32.58</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>71.84</v>
+        <v>75.38</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>43.49</v>
+        <v>41.06</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>26.21</v>
+        <v>25.43</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>64.05</v>
+        <v>61.1</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.1</v>
+        <v>50.6</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>29.28</v>
+        <v>28.27</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>70.06</v>
+        <v>71.08</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>36.85</v>
+        <v>38.78</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>62.67</v>
+        <v>66.31</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>39.34</v>
+        <v>39.8</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>27.35</v>
+        <v>26.69</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>59.81</v>
+        <v>59.42</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>29.3</v>
+        <v>28.84</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>59.18</v>
+        <v>57.02</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>47.54</v>
+        <v>45.17</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.53</v>
+        <v>26.89</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>69.12</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>47.77</v>
+        <v>45.02</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>27.42</v>
+        <v>24.63</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>76.81999999999999</v>
+        <v>74.06999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46.75</v>
+        <v>43.42</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>25.61</v>
+        <v>23.97</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>70.55</v>
+        <v>71.11</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.48</v>
+        <v>22.42</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>53.08</v>
+        <v>55.51</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.25</v>
+        <v>22.72</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.72</v>
+        <v>55.15</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>54.92</v>
+        <v>52.76</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>28.83</v>
+        <v>24.99</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>77.59999999999999</v>
+        <v>75.15000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>30.76</v>
+        <v>32.57</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>58.58</v>
+        <v>62.25</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>37.91</v>
+        <v>41.78</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>63.95</v>
+        <v>66.23</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>38.1</v>
+        <v>37.26</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>66</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47.69</v>
+        <v>48.46</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>30.46</v>
+        <v>30.81</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>65.87</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>47.25</v>
+        <v>45.38</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>29.6</v>
+        <v>26.44</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>68.52</v>
+        <v>67.28</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>15.14</v>
+        <v>18.33</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>48.38</v>
+        <v>60.62</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>45.23</v>
+        <v>47.61</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.96</v>
+        <v>28.08</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>65.22</v>
+        <v>70.65000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46.56</v>
+        <v>43.16</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.05</v>
+        <v>25.09</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>72.72</v>
+        <v>69.7</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.91</v>
+        <v>14.92</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.78</v>
+        <v>59.04</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>52.32</v>
+        <v>57.73</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>38.35</v>
+        <v>38.56</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>64.17</v>
+        <v>69.59</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.51</v>
+        <v>9.26</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.94</v>
+        <v>54.75</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.61</v>
+        <v>10.51</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>52.13</v>
+        <v>45.96</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>49.7</v>
+        <v>47.93</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>30.63</v>
+        <v>31.13</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>75.09999999999999</v>
+        <v>74.88</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>17.64</v>
+        <v>17.84</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>48.18</v>
+        <v>48.17</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,20 +1700,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>51.32</v>
+        <v>45.39</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>28.99</v>
+        <v>27.84</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>75.63</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.16</v>
+        <v>46.22</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.1</v>
+        <v>26.78</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.3</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>34.17</v>
+        <v>32.95</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>79.39</v>
+        <v>75.87</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>29.23</v>
+        <v>27.84</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>62.13</v>
+        <v>58.14</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>49.38</v>
+        <v>51.55</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>33.12</v>
+        <v>31.39</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>68.31999999999999</v>
+        <v>69.84</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>47.71</v>
+        <v>58.62</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>33.09</v>
+        <v>43.83</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.27</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>298407</v>
+        <v>314404</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>16.73</v>
+        <v>17.63</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1192244</v>
+        <v>1159316</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>66.86</v>
+        <v>65.01000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>291952</v>
+        <v>308745</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>16.37</v>
+        <v>17.31</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>628</v>
+        <v>766</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.04</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-01
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-30.tif</t>
+          <t>fli_fars_2026-10-01.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>93.19</v>
+        <v>88.59</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>36.46</v>
+        <v>35.15</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52.13</v>
+        <v>52.45</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.95</v>
+        <v>27.66</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>78.31</v>
+        <v>79.31999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46.74</v>
+        <v>49.49</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>26.66</v>
+        <v>27.42</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>79.23999999999999</v>
+        <v>83.88</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.58</v>
+        <v>18.33</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>69.39</v>
+        <v>68.08</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>50.08</v>
+        <v>50.56</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.58</v>
+        <v>35.14</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>75.38</v>
+        <v>76.59</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>41.06</v>
+        <v>41.89</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>25.43</v>
+        <v>26.39</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>61.1</v>
+        <v>61.13</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.6</v>
+        <v>47.97</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>28.27</v>
+        <v>26.28</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>71.08</v>
+        <v>70.42</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.78</v>
+        <v>34.62</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>66.31</v>
+        <v>60</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>39.8</v>
+        <v>43.42</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>26.69</v>
+        <v>28.95</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>59.42</v>
+        <v>64</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>28.84</v>
+        <v>27.37</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>57.02</v>
+        <v>58.68</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.17</v>
+        <v>45.66</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.89</v>
+        <v>26.76</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.01000000000001</v>
+        <v>66.86</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.02</v>
+        <v>44.12</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>24.63</v>
+        <v>25.87</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.06999999999999</v>
+        <v>71.36</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>43.42</v>
+        <v>40.88</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>23.97</v>
+        <v>21.94</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>71.11</v>
+        <v>68.48</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.42</v>
+        <v>20.44</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>55.51</v>
+        <v>51.55</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.72</v>
+        <v>21.25</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>55.15</v>
+        <v>54.26</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.76</v>
+        <v>53.97</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>24.99</v>
+        <v>26.74</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.15000000000001</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>32.57</v>
+        <v>26.69</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>62.25</v>
+        <v>53.76</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>41.78</v>
+        <v>39.83</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>66.23</v>
+        <v>63.64</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.26</v>
+        <v>33.69</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>64.51000000000001</v>
+        <v>60.21</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>48.46</v>
+        <v>48.68</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>30.81</v>
+        <v>30.98</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>67.20999999999999</v>
+        <v>66.84</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>45.38</v>
+        <v>44.86</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.44</v>
+        <v>26.31</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>67.28</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>18.33</v>
+        <v>16.08</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>60.62</v>
+        <v>52.16</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.61</v>
+        <v>46.46</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.08</v>
+        <v>30.51</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>70.65000000000001</v>
+        <v>67.76000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.16</v>
+        <v>43.74</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.09</v>
+        <v>28.03</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>69.7</v>
+        <v>69.94</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.92</v>
+        <v>14.03</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>59.04</v>
+        <v>54.85</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>57.73</v>
+        <v>49.58</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>38.56</v>
+        <v>32.58</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>69.59</v>
+        <v>61</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.26</v>
+        <v>10.29</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.75</v>
+        <v>57.64</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.51</v>
+        <v>12.08</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>45.96</v>
+        <v>52.18</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>47.93</v>
+        <v>49.76</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>31.13</v>
+        <v>33.21</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>74.88</v>
+        <v>76.72</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>17.84</v>
+        <v>18.22</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>48.17</v>
+        <v>49.31</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>45.39</v>
+        <v>48.48</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27.84</v>
+        <v>28.82</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>69.01000000000001</v>
+        <v>73.37</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46.22</v>
+        <v>45.23</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.78</v>
+        <v>26.69</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.45999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.95</v>
+        <v>32.91</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>75.87</v>
+        <v>78.58</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>27.84</v>
+        <v>27.88</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>58.14</v>
+        <v>59.77</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>51.55</v>
+        <v>47.12</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>31.39</v>
+        <v>30.31</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>69.84</v>
+        <v>64.05</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>58.62</v>
+        <v>56.71</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>43.83</v>
+        <v>38.74</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>73.51000000000001</v>
+        <v>72.22</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>314404</v>
+        <v>351333</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.63</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1159316</v>
+        <v>1177259</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>65.01000000000001</v>
+        <v>66.02</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>308745</v>
+        <v>254060</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>17.31</v>
+        <v>14.25</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>766</v>
+        <v>579</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-02
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-01.tif</t>
+          <t>fli_fars_2026-10-02.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>88.59</v>
+        <v>87.18000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>35.15</v>
+        <v>34.17</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>52.45</v>
+        <v>51.55</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>27.66</v>
+        <v>26.82</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>79.31999999999999</v>
+        <v>78.19</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>49.49</v>
+        <v>48.19</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>27.42</v>
+        <v>27.7</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>83.88</v>
+        <v>78.81999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.33</v>
+        <v>17.2</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>68.08</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,20 +800,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>50.56</v>
+        <v>39.83</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>35.14</v>
+        <v>24.11</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>76.59</v>
+        <v>63.78</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>41.89</v>
+        <v>40.01</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>26.39</v>
+        <v>25.49</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>61.13</v>
+        <v>59.39</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>47.97</v>
+        <v>50.58</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>26.28</v>
+        <v>28.83</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>70.42</v>
+        <v>70.36</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.62</v>
+        <v>31.54</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>60</v>
+        <v>54.44</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>43.42</v>
+        <v>36.25</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>28.95</v>
+        <v>25.52</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>64</v>
+        <v>55.14</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>27.37</v>
+        <v>26.9</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>58.68</v>
+        <v>60.99</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.66</v>
+        <v>45.93</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.76</v>
+        <v>28.24</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.86</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.12</v>
+        <v>44.79</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.87</v>
+        <v>25.54</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>71.36</v>
+        <v>73.62</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>40.88</v>
+        <v>39.2</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>21.94</v>
+        <v>20.44</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>68.48</v>
+        <v>66.59</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.44</v>
+        <v>20.2</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>51.55</v>
+        <v>50.06</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.25</v>
+        <v>21.32</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>54.26</v>
+        <v>52.27</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>53.97</v>
+        <v>54.15</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>26.74</v>
+        <v>29.18</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>77.18000000000001</v>
+        <v>76.89</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.69</v>
+        <v>27.48</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53.76</v>
+        <v>56.08</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>39.83</v>
+        <v>37.78</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>63.64</v>
+        <v>61.18</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>33.69</v>
+        <v>35.49</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>60.21</v>
+        <v>60.75</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>48.68</v>
+        <v>49.27</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>30.98</v>
+        <v>29.97</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.84</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>44.86</v>
+        <v>47.06</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.31</v>
+        <v>28.8</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>67.54000000000001</v>
+        <v>68.09</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>16.08</v>
+        <v>14.75</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>52.16</v>
+        <v>46.27</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46.46</v>
+        <v>48.86</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>30.51</v>
+        <v>28.31</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>67.76000000000001</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.74</v>
+        <v>43.98</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.03</v>
+        <v>25.15</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>69.94</v>
+        <v>67.73</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.03</v>
+        <v>14.19</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>54.85</v>
+        <v>53.92</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>49.58</v>
+        <v>50.96</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.58</v>
+        <v>36.73</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>61</v>
+        <v>62.56</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>10.29</v>
+        <v>9.07</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>57.64</v>
+        <v>52.01</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>12.08</v>
+        <v>11.23</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>52.18</v>
+        <v>51.19</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>49.76</v>
+        <v>46.67</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>33.21</v>
+        <v>23.24</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>76.72</v>
+        <v>72.25</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>18.22</v>
+        <v>17.41</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>49.31</v>
+        <v>50.51</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>48.48</v>
+        <v>46.72</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>28.82</v>
+        <v>27.39</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>73.37</v>
+        <v>71.92</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.23</v>
+        <v>46.28</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.69</v>
+        <v>27.28</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.5</v>
+        <v>66.12</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.91</v>
+        <v>31.86</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>78.58</v>
+        <v>73.81999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>27.88</v>
+        <v>26.85</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>59.77</v>
+        <v>56.53</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>47.12</v>
+        <v>49.4</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>30.31</v>
+        <v>32.15</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>64.05</v>
+        <v>68.5</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>56.71</v>
+        <v>46.36</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>38.74</v>
+        <v>32.47</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>72.22</v>
+        <v>62.73</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>351333</v>
+        <v>337924</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.7</v>
+        <v>18.95</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1177259</v>
+        <v>1248121</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>66.02</v>
+        <v>69.98999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>254060</v>
+        <v>196771</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>14.25</v>
+        <v>11.03</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>579</v>
+        <v>415</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-03
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-02.tif</t>
+          <t>fli_fars_2026-10-03.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>87.18000000000001</v>
+        <v>86.43000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.17</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>51.55</v>
+        <v>51.45</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.82</v>
+        <v>26.47</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>78.19</v>
+        <v>76.97</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>48.19</v>
+        <v>44.97</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>27.7</v>
+        <v>21.88</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>78.81999999999999</v>
+        <v>77.06999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>17.2</v>
+        <v>19.02</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>66.43000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.83</v>
+        <v>39.84</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>24.11</v>
+        <v>24.15</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>63.78</v>
+        <v>64.78</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>40.01</v>
+        <v>40.86</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>25.49</v>
+        <v>23.74</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.39</v>
+        <v>62.15</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.58</v>
+        <v>51.85</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>28.83</v>
+        <v>26.2</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>70.36</v>
+        <v>74.61</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>31.54</v>
+        <v>32.11</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>54.44</v>
+        <v>56.33</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>36.25</v>
+        <v>39.98</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>25.52</v>
+        <v>28.27</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>55.14</v>
+        <v>60.1</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>26.9</v>
+        <v>28.26</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>60.99</v>
+        <v>61.86</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.93</v>
+        <v>45.97</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.24</v>
+        <v>27.84</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.15000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.79</v>
+        <v>45.28</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.54</v>
+        <v>25.75</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.62</v>
+        <v>74.44</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>39.2</v>
+        <v>41.52</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>20.44</v>
+        <v>21.94</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>66.59</v>
+        <v>67.48</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.2</v>
+        <v>20.39</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>50.06</v>
+        <v>48.6</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.32</v>
+        <v>21.63</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>52.27</v>
+        <v>56.37</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>54.15</v>
+        <v>54.64</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>29.18</v>
+        <v>29.28</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>76.89</v>
+        <v>76.7</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.48</v>
+        <v>26.79</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.08</v>
+        <v>55.47</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>37.78</v>
+        <v>39.78</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>61.18</v>
+        <v>62.31</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>35.49</v>
+        <v>34.85</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>60.75</v>
+        <v>61.3</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>49.27</v>
+        <v>50.81</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>29.97</v>
+        <v>33.49</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>68.26000000000001</v>
+        <v>68.06</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>47.06</v>
+        <v>45.25</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>28.8</v>
+        <v>28.13</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>68.09</v>
+        <v>66.33</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14.75</v>
+        <v>15.98</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>46.27</v>
+        <v>51.54</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.86</v>
+        <v>48.65</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.31</v>
+        <v>26.95</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>69.68000000000001</v>
+        <v>68.69</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.98</v>
+        <v>43.61</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.15</v>
+        <v>24.61</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.73</v>
+        <v>69.59</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.19</v>
+        <v>14.79</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>53.92</v>
+        <v>57.87</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>50.96</v>
+        <v>52.19</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>36.73</v>
+        <v>35.51</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>62.56</v>
+        <v>63.57</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.07</v>
+        <v>8.82</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>52.01</v>
+        <v>51.24</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.23</v>
+        <v>10.09</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>51.19</v>
+        <v>47.17</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>46.67</v>
+        <v>45.62</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>23.24</v>
+        <v>26.14</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>72.25</v>
+        <v>71.73</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>17.41</v>
+        <v>18.59</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>50.51</v>
+        <v>50.63</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.72</v>
+        <v>46.24</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27.39</v>
+        <v>29.21</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>71.92</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46.28</v>
+        <v>47.12</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.28</v>
+        <v>26.48</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.12</v>
+        <v>69.05</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>31.86</v>
+        <v>32.66</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.81999999999999</v>
+        <v>75.98</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>26.85</v>
+        <v>27.84</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>56.53</v>
+        <v>60.26</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>49.4</v>
+        <v>48.66</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>32.15</v>
+        <v>32.77</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>68.5</v>
+        <v>66.5</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>46.36</v>
+        <v>52.2</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>32.47</v>
+        <v>38.56</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.73</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>337924</v>
+        <v>346221</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.95</v>
+        <v>19.42</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1248121</v>
+        <v>1245844</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>69.98999999999999</v>
+        <v>69.86</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>196771</v>
+        <v>190920</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>11.03</v>
+        <v>10.71</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>415</v>
+        <v>246</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-04
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -68,12 +68,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E53935"/>
+        <fgColor rgb="00C7A900"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C7A900"/>
+        <fgColor rgb="00E53935"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,10 +119,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-03.tif</t>
+          <t>fli_fars_2026-10-04.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>86.43000000000001</v>
+        <v>84.03</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>33.96</v>
+        <v>33.47</v>
       </c>
     </row>
     <row r="10">
@@ -704,20 +704,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>51.45</v>
+        <v>47.68</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.47</v>
+        <v>22.71</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>76.97</v>
+        <v>74.95</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -736,18 +736,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.97</v>
+        <v>44.01</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>21.88</v>
+        <v>22.79</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>77.06999999999999</v>
+        <v>75.97</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -768,18 +768,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>19.02</v>
+        <v>18.26</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>74.5</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -800,18 +800,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.84</v>
+        <v>42.21</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>24.15</v>
+        <v>27.54</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>64.78</v>
+        <v>68.86</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -832,18 +832,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>40.86</v>
+        <v>40.05</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>23.74</v>
+        <v>24.72</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>62.15</v>
+        <v>59.59</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.85</v>
+        <v>48.86</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>26.2</v>
+        <v>29.92</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>74.61</v>
+        <v>72.73999999999999</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -896,18 +896,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>32.11</v>
+        <v>33.94</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>56.33</v>
+        <v>59.62</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -928,18 +928,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>39.98</v>
+        <v>38.36</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>28.27</v>
+        <v>26.7</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>60.1</v>
+        <v>59.34</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -960,18 +960,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>28.26</v>
+        <v>25.88</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>61.86</v>
+        <v>55.89</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -992,18 +992,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.97</v>
+        <v>42.32</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.84</v>
+        <v>24.54</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.8</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1024,18 +1024,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.28</v>
+        <v>43.71</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.75</v>
+        <v>24.57</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.44</v>
+        <v>72.88</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1056,18 +1056,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>41.52</v>
+        <v>39.54</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>21.94</v>
+        <v>23.5</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>67.48</v>
+        <v>66.88</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1088,18 +1088,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.39</v>
+        <v>24.07</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.6</v>
+        <v>57.18</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1120,18 +1120,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.63</v>
+        <v>21.97</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.37</v>
+        <v>55.53</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1152,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>54.64</v>
+        <v>49.94</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>29.28</v>
+        <v>23.86</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>76.7</v>
+        <v>71.89</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1184,18 +1184,18 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.79</v>
+        <v>28.82</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>55.47</v>
+        <v>57.33</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1216,18 +1216,18 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>39.78</v>
+        <v>36.56</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>62.31</v>
+        <v>62.45</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1248,18 +1248,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>34.85</v>
+        <v>33.97</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>61.3</v>
+        <v>59.32</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>50.81</v>
+        <v>46.61</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>33.49</v>
+        <v>28.25</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>68.06</v>
+        <v>66.11</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,18 +1312,18 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>45.25</v>
+        <v>42.85</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>28.13</v>
+        <v>24.57</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>66.33</v>
+        <v>65.13</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1344,18 +1344,18 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>15.98</v>
+        <v>14.65</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>51.54</v>
+        <v>47.82</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1444,18 +1444,18 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.65</v>
+        <v>42.23</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.95</v>
+        <v>25.63</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>68.69</v>
+        <v>63.06</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1476,18 +1476,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.61</v>
+        <v>42.84</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>24.61</v>
+        <v>25.79</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>69.59</v>
+        <v>67.97</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1508,18 +1508,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.79</v>
+        <v>16.28</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>57.87</v>
+        <v>65.27</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1540,20 +1540,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>52.19</v>
+        <v>47.38</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>35.51</v>
+        <v>31.21</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>63.57</v>
+        <v>58.79</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1572,18 +1572,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.82</v>
+        <v>9.24</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>51.24</v>
+        <v>53.5</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1604,18 +1604,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.09</v>
+        <v>10.7</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>47.17</v>
+        <v>46.97</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1636,18 +1636,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>45.62</v>
+        <v>44.77</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>26.14</v>
+        <v>26.64</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.73</v>
+        <v>75.66</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1668,18 +1668,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>18.59</v>
+        <v>18.06</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>50.63</v>
+        <v>48.58</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1700,18 +1700,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.24</v>
+        <v>43.4</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>29.21</v>
+        <v>25.38</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>69.06999999999999</v>
+        <v>67.83</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1732,18 +1732,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>47.12</v>
+        <v>48.6</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.48</v>
+        <v>27.36</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>69.05</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1764,18 +1764,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.66</v>
+        <v>30.06</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>75.98</v>
+        <v>74.26000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>27.84</v>
+        <v>24.94</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>60.26</v>
+        <v>55.42</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1828,18 +1828,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>48.66</v>
+        <v>45.25</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>32.77</v>
+        <v>28.2</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>66.5</v>
+        <v>62.72</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>52.2</v>
+        <v>49.31</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>38.56</v>
+        <v>35.16</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>67.73999999999999</v>
+        <v>65.16</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>خیلی زیاد</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1940,14 +1940,14 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>346221</v>
+        <v>345778</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.42</v>
+        <v>19.39</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1959,14 +1959,14 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1245844</v>
+        <v>1289071</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>69.86</v>
+        <v>72.29000000000001</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>خیلی زیاد</t>
         </is>
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>190920</v>
+        <v>148272</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>10.71</v>
+        <v>8.31</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>246</v>
+        <v>110</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-06
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-04.tif</t>
+          <t>fli_fars_2026-10-06.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>84.03</v>
+        <v>85.95</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>33.47</v>
+        <v>33.62</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.68</v>
+        <v>49.52</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>22.71</v>
+        <v>24.73</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>74.95</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.01</v>
+        <v>47.07</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>22.79</v>
+        <v>25.43</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>75.97</v>
+        <v>78.22</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.26</v>
+        <v>16.45</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>69.31999999999999</v>
+        <v>63.3</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>42.21</v>
+        <v>44.41</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.54</v>
+        <v>29.85</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>68.86</v>
+        <v>71.58</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>40.05</v>
+        <v>39.62</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>24.72</v>
+        <v>23.12</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.59</v>
+        <v>60.07</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>48.86</v>
+        <v>48.33</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>29.92</v>
+        <v>27.36</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>72.73999999999999</v>
+        <v>68.13</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.94</v>
+        <v>34.02</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>59.62</v>
+        <v>58.38</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>38.36</v>
+        <v>35.92</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>26.7</v>
+        <v>25.73</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>59.34</v>
+        <v>55.66</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>25.88</v>
+        <v>24.32</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>55.89</v>
+        <v>56.41</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.32</v>
+        <v>43.9</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>24.54</v>
+        <v>26.21</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>64.09999999999999</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>43.71</v>
+        <v>45.28</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>24.57</v>
+        <v>26.53</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.88</v>
+        <v>73.05</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>39.54</v>
+        <v>45.26</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>23.5</v>
+        <v>22.55</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>66.88</v>
+        <v>69.43000000000001</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>24.07</v>
+        <v>22.45</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>57.18</v>
+        <v>50.65</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.97</v>
+        <v>24.59</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>55.53</v>
+        <v>60.86</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>49.94</v>
+        <v>51.7</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>23.86</v>
+        <v>27.19</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>71.89</v>
+        <v>75.03</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.82</v>
+        <v>27.6</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>57.33</v>
+        <v>53.96</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>36.56</v>
+        <v>32.98</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>62.45</v>
+        <v>55.96</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>33.97</v>
+        <v>35.5</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>59.32</v>
+        <v>61.48</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46.61</v>
+        <v>47.24</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>28.25</v>
+        <v>27.67</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.11</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>42.85</v>
+        <v>44.52</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>24.57</v>
+        <v>26.93</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>65.13</v>
+        <v>64.52</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14.65</v>
+        <v>13.85</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>47.82</v>
+        <v>42.46</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.23</v>
+        <v>44.93</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.63</v>
+        <v>25.95</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>63.06</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>42.84</v>
+        <v>43.97</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.79</v>
+        <v>25.63</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.97</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.28</v>
+        <v>16.1</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>65.27</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>47.38</v>
+        <v>40.85</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>31.21</v>
+        <v>25.79</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>58.79</v>
+        <v>51.9</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.24</v>
+        <v>8.57</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>53.5</v>
+        <v>51.19</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.7</v>
+        <v>10.45</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46.97</v>
+        <v>47.7</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>44.77</v>
+        <v>44.93</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>26.64</v>
+        <v>26.28</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>75.66</v>
+        <v>71.61</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>18.06</v>
+        <v>16.3</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>48.58</v>
+        <v>43.27</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>43.4</v>
+        <v>44.49</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>25.38</v>
+        <v>24.07</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>67.83</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>48.6</v>
+        <v>45.77</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.36</v>
+        <v>25.14</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>70.98999999999999</v>
+        <v>67.41</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>30.06</v>
+        <v>30.2</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.26000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.94</v>
+        <v>25.26</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.42</v>
+        <v>53.45</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>45.25</v>
+        <v>41.77</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>28.2</v>
+        <v>23.48</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>62.72</v>
+        <v>59.45</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>49.31</v>
+        <v>45.78</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>35.16</v>
+        <v>31.3</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>65.16</v>
+        <v>62.66</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>345778</v>
+        <v>348429</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.39</v>
+        <v>19.54</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1289071</v>
+        <v>1261727</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>72.29000000000001</v>
+        <v>70.76000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>148272</v>
+        <v>172939</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>8.31</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-08
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-06.tif</t>
+          <t>fli_fars_2026-10-08.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>85.95</v>
+        <v>85.05</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>33.62</v>
+        <v>34.48</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>49.52</v>
+        <v>49.95</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>24.73</v>
+        <v>25.3</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>76.45999999999999</v>
+        <v>78.09</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>47.07</v>
+        <v>46.22</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.43</v>
+        <v>24.8</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>78.22</v>
+        <v>77</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.45</v>
+        <v>16.43</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.3</v>
+        <v>62.04</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44.41</v>
+        <v>45.09</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>29.85</v>
+        <v>30.73</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>71.58</v>
+        <v>71.73999999999999</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -835,10 +835,10 @@
         <v>39.62</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>23.12</v>
+        <v>22.12</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>60.07</v>
+        <v>60.92</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>48.33</v>
+        <v>53.38</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>27.36</v>
+        <v>34.77</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>68.13</v>
+        <v>75.55</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.02</v>
+        <v>34.89</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>58.38</v>
+        <v>59.19</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>35.92</v>
+        <v>35.54</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>25.73</v>
+        <v>24.62</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>55.66</v>
+        <v>55.23</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>24.32</v>
+        <v>24.92</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>56.41</v>
+        <v>59.51</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>43.9</v>
+        <v>44.82</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.21</v>
+        <v>26.65</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>64.79000000000001</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.28</v>
+        <v>46.5</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>26.53</v>
+        <v>27.3</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.05</v>
+        <v>75.92</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>45.26</v>
+        <v>44.91</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>22.55</v>
+        <v>24.39</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>69.43000000000001</v>
+        <v>70.01000000000001</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.45</v>
+        <v>22.69</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>50.65</v>
+        <v>54.91</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>24.59</v>
+        <v>23.34</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>60.86</v>
+        <v>60.11</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>51.7</v>
+        <v>53.42</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>27.19</v>
+        <v>28.83</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.03</v>
+        <v>75.23</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.6</v>
+        <v>28.91</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53.96</v>
+        <v>58.25</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>32.98</v>
+        <v>35.47</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>55.96</v>
+        <v>60.6</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>35.5</v>
+        <v>36.02</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>61.48</v>
+        <v>62.91</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47.24</v>
+        <v>52.7</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>27.67</v>
+        <v>34.86</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.29000000000001</v>
+        <v>70.62</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>44.52</v>
+        <v>45.81</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.93</v>
+        <v>27.32</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>64.52</v>
+        <v>66.14</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.85</v>
+        <v>13.61</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>42.46</v>
+        <v>42.4</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>44.93</v>
+        <v>47.24</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.95</v>
+        <v>28.6</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>67.15000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.97</v>
+        <v>44.37</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.63</v>
+        <v>26.17</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>69.06999999999999</v>
+        <v>69.97</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.1</v>
+        <v>16.41</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>64.04000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>40.85</v>
+        <v>47.39</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>25.79</v>
+        <v>32.67</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>51.9</v>
+        <v>58.5</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.57</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>51.19</v>
+        <v>50.8</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.45</v>
+        <v>10.22</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>47.7</v>
+        <v>48.38</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>44.93</v>
+        <v>44.27</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>26.28</v>
+        <v>24.38</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.61</v>
+        <v>71.69</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>16.3</v>
+        <v>16.6</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>43.27</v>
+        <v>44.34</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>44.49</v>
+        <v>46.43</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>24.07</v>
+        <v>28.14</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>69.01000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.77</v>
+        <v>48.45</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.14</v>
+        <v>29.68</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.41</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>30.2</v>
+        <v>31.04</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>71.8</v>
+        <v>75.62</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>25.26</v>
+        <v>26.26</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>53.45</v>
+        <v>57.03</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>41.77</v>
+        <v>46.29</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>23.48</v>
+        <v>28.03</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>59.45</v>
+        <v>62.9</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>45.78</v>
+        <v>48.59</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>31.3</v>
+        <v>33.97</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.66</v>
+        <v>63.15</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>348429</v>
+        <v>325582</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.54</v>
+        <v>18.26</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1261727</v>
+        <v>1255808</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>70.76000000000001</v>
+        <v>70.42</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>172939</v>
+        <v>201672</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>9.699999999999999</v>
+        <v>11.31</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-09
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-08.tif</t>
+          <t>fli_fars_2026-10-09.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>85.05</v>
+        <v>85.12</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.48</v>
+        <v>34.91</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>49.95</v>
+        <v>49.68</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>78.09</v>
+        <v>79.12</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46.22</v>
+        <v>46.81</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>24.8</v>
+        <v>25.72</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>77</v>
+        <v>77.47</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.43</v>
+        <v>16.13</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>62.04</v>
+        <v>59.96</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>45.09</v>
+        <v>47.1</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.73</v>
+        <v>33.2</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>71.73999999999999</v>
+        <v>74.16</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>39.62</v>
+        <v>39.23</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>22.12</v>
+        <v>23.32</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>60.92</v>
+        <v>59.17</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>53.38</v>
+        <v>51.13</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>34.77</v>
+        <v>30.23</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>75.55</v>
+        <v>75.27</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.89</v>
+        <v>35.88</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>59.19</v>
+        <v>60.82</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>35.54</v>
+        <v>35.48</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>24.62</v>
+        <v>25.11</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>55.23</v>
+        <v>54.74</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>24.92</v>
+        <v>25.04</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>59.51</v>
+        <v>58.44</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>44.82</v>
+        <v>42.98</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>26.65</v>
+        <v>25.95</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.79000000000001</v>
+        <v>64.77</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46.5</v>
+        <v>44.65</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>27.3</v>
+        <v>25.03</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>75.92</v>
+        <v>73.56</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.91</v>
+        <v>44.63</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>24.39</v>
+        <v>24.06</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>70.01000000000001</v>
+        <v>68.64</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.69</v>
+        <v>23.6</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>54.91</v>
+        <v>55.95</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.34</v>
+        <v>23.59</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>60.11</v>
+        <v>58.32</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>53.42</v>
+        <v>52.41</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>28.83</v>
+        <v>27.58</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>75.23</v>
+        <v>74.75</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.91</v>
+        <v>32.25</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>58.25</v>
+        <v>63.13</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>35.47</v>
+        <v>33.92</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>60.6</v>
+        <v>59.96</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>36.02</v>
+        <v>40.31</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>62.91</v>
+        <v>69</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,20 +1280,20 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>52.7</v>
+        <v>47.9</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>34.86</v>
+        <v>31.16</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>70.62</v>
+        <v>65.19</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>45.81</v>
+        <v>44.66</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>27.32</v>
+        <v>26.93</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>66.14</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.61</v>
+        <v>13.84</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>42.4</v>
+        <v>44.32</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.24</v>
+        <v>47.59</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.6</v>
+        <v>29.22</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>69.59999999999999</v>
+        <v>70.11</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.37</v>
+        <v>42.52</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>26.17</v>
+        <v>25.93</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>69.97</v>
+        <v>68.33</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.41</v>
+        <v>15.96</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>65.09999999999999</v>
+        <v>63.73</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>47.39</v>
+        <v>49.28</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.67</v>
+        <v>35.04</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>58.5</v>
+        <v>60.86</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.800000000000001</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>50.8</v>
+        <v>52.15</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.22</v>
+        <v>10.06</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>48.38</v>
+        <v>45.07</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>44.27</v>
+        <v>45.09</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>24.38</v>
+        <v>25.59</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.69</v>
+        <v>71.92</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>16.6</v>
+        <v>15.69</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>44.34</v>
+        <v>41.05</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46.43</v>
+        <v>47.92</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>28.14</v>
+        <v>30.37</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>68.40000000000001</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>48.45</v>
+        <v>45.94</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>29.68</v>
+        <v>27.22</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>70.29000000000001</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>31.04</v>
+        <v>29.97</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>75.62</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>26.26</v>
+        <v>24.98</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>57.03</v>
+        <v>55.93</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46.29</v>
+        <v>47.06</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>28.03</v>
+        <v>29.79</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>62.9</v>
+        <v>63.8</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>48.59</v>
+        <v>52.18</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>33.97</v>
+        <v>38.98</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>63.15</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>325582</v>
+        <v>325078</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.26</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1255808</v>
+        <v>1240415</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>70.42</v>
+        <v>69.56</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>201672</v>
+        <v>217563</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>11.31</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-11
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-09.tif</t>
+          <t>fli_fars_2026-10-11.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>85.12</v>
+        <v>85.86</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.91</v>
+        <v>34.63</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>49.68</v>
+        <v>48.42</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.5</v>
+        <v>24.75</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>79.12</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46.81</v>
+        <v>47.04</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.72</v>
+        <v>26.23</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>77.47</v>
+        <v>79.56999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.13</v>
+        <v>16.24</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>59.96</v>
+        <v>61.14</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>47.1</v>
+        <v>48.59</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>33.2</v>
+        <v>33.68</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>74.16</v>
+        <v>74.13</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>39.23</v>
+        <v>40.84</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>23.32</v>
+        <v>22.96</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.17</v>
+        <v>62</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.13</v>
+        <v>50.1</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>30.23</v>
+        <v>27.16</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>75.27</v>
+        <v>71.38</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>35.88</v>
+        <v>38.64</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>60.82</v>
+        <v>66.7</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>35.48</v>
+        <v>36.82</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>25.11</v>
+        <v>26.54</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>54.74</v>
+        <v>56.73</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>25.04</v>
+        <v>24.51</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>58.44</v>
+        <v>57.38</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.98</v>
+        <v>44.55</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.95</v>
+        <v>27.37</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>64.77</v>
+        <v>65.05</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.65</v>
+        <v>45.56</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.03</v>
+        <v>25.12</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.56</v>
+        <v>73.54000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.63</v>
+        <v>47.25</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>24.06</v>
+        <v>28.75</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>68.64</v>
+        <v>72.79000000000001</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.6</v>
+        <v>23.9</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>55.95</v>
+        <v>58.05</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.59</v>
+        <v>24.93</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.32</v>
+        <v>61.25</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.41</v>
+        <v>51.77</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>27.58</v>
+        <v>26.93</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>74.75</v>
+        <v>73.98</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>32.25</v>
+        <v>31.48</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>63.13</v>
+        <v>61.98</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>33.92</v>
+        <v>32.92</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>59.96</v>
+        <v>55.39</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>40.31</v>
+        <v>37.37</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>69</v>
+        <v>63.73</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47.9</v>
+        <v>49.37</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>31.16</v>
+        <v>31.93</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>65.19</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>44.66</v>
+        <v>44.4</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.93</v>
+        <v>26.91</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>64.70999999999999</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.84</v>
+        <v>13.59</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>44.32</v>
+        <v>42.14</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.59</v>
+        <v>42.6</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>29.22</v>
+        <v>24.21</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>70.11</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>42.52</v>
+        <v>43.36</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.93</v>
+        <v>26.9</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>68.33</v>
+        <v>67.23</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.96</v>
+        <v>16.14</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.73</v>
+        <v>65.78</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>49.28</v>
+        <v>42.03</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>35.04</v>
+        <v>27.91</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>60.86</v>
+        <v>53.73</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.710000000000001</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>52.15</v>
+        <v>60.48</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.06</v>
+        <v>11.24</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>45.07</v>
+        <v>49.34</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>45.09</v>
+        <v>43.28</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>25.59</v>
+        <v>27.06</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.92</v>
+        <v>71.73999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>15.69</v>
+        <v>16.15</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>41.05</v>
+        <v>42.47</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>47.92</v>
+        <v>44.31</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>30.37</v>
+        <v>25.72</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>70.23999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.94</v>
+        <v>45.42</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.22</v>
+        <v>25.65</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>67.51000000000001</v>
+        <v>66.78</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>29.97</v>
+        <v>30.09</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.84999999999999</v>
+        <v>72.55</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.98</v>
+        <v>25.26</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.93</v>
+        <v>53.88</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>47.06</v>
+        <v>40.69</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>29.79</v>
+        <v>23.44</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>63.8</v>
+        <v>58.3</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,20 +1860,20 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>52.18</v>
+        <v>45.62</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>38.98</v>
+        <v>32.35</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>68.18000000000001</v>
+        <v>61.88</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>325078</v>
+        <v>349008</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.23</v>
+        <v>19.57</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1240415</v>
+        <v>1218722</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>69.56</v>
+        <v>68.34</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>217563</v>
+        <v>215334</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>12.2</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-12
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-11.tif</t>
+          <t>fli_fars_2026-10-12.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>85.86</v>
+        <v>83.05</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.63</v>
+        <v>34.16</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.42</v>
+        <v>48.64</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>24.75</v>
+        <v>26.06</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>76.59999999999999</v>
+        <v>75.14</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>47.04</v>
+        <v>45.97</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>26.23</v>
+        <v>23.92</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>79.56999999999999</v>
+        <v>77.61</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.24</v>
+        <v>15.57</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>61.14</v>
+        <v>58.88</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>48.59</v>
+        <v>44.2</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>33.68</v>
+        <v>29.93</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>74.13</v>
+        <v>69.48</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>40.84</v>
+        <v>42.99</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>22.96</v>
+        <v>27.78</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>62</v>
+        <v>62.42</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.1</v>
+        <v>54.55</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>27.16</v>
+        <v>33.89</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>71.38</v>
+        <v>74.66</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.64</v>
+        <v>34.93</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>66.7</v>
+        <v>59.93</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>36.82</v>
+        <v>35.27</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>26.54</v>
+        <v>25.04</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>56.73</v>
+        <v>54.93</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>24.51</v>
+        <v>25.27</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>57.38</v>
+        <v>57.01</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>44.55</v>
+        <v>44.46</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.37</v>
+        <v>28.55</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>65.05</v>
+        <v>63.97</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45.56</v>
+        <v>46.88</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.12</v>
+        <v>25.93</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.54000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>47.25</v>
+        <v>44.42</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>28.75</v>
+        <v>26.95</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>72.79000000000001</v>
+        <v>69.41</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>23.9</v>
+        <v>22.9</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>58.05</v>
+        <v>56.06</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>24.93</v>
+        <v>23.35</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>61.25</v>
+        <v>58.32</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>51.77</v>
+        <v>52.22</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>26.93</v>
+        <v>27.99</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>73.98</v>
+        <v>73.47</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>31.48</v>
+        <v>28.24</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>61.98</v>
+        <v>56.77</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>32.92</v>
+        <v>31.84</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>55.39</v>
+        <v>56.72</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.37</v>
+        <v>37.22</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>63.73</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>49.37</v>
+        <v>49.12</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>31.93</v>
+        <v>32.33</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>67.26000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>44.4</v>
+        <v>44.01</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.91</v>
+        <v>26.18</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>64.56999999999999</v>
+        <v>65.14</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.59</v>
+        <v>14.25</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>42.14</v>
+        <v>45.57</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.6</v>
+        <v>42.43</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>24.21</v>
+        <v>25.88</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>64.20999999999999</v>
+        <v>63.6</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.36</v>
+        <v>45.83</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>26.9</v>
+        <v>28.57</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.23</v>
+        <v>71.67</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.14</v>
+        <v>15.26</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>65.78</v>
+        <v>60.21</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>42.03</v>
+        <v>46.06</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.91</v>
+        <v>30.74</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>53.73</v>
+        <v>57.16</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.210000000000001</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>60.48</v>
+        <v>58.48</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.24</v>
+        <v>10.98</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>49.34</v>
+        <v>47.65</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>43.28</v>
+        <v>41.74</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>27.06</v>
+        <v>25.39</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.73999999999999</v>
+        <v>71.75</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>16.15</v>
+        <v>15.54</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>42.47</v>
+        <v>41.27</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>44.31</v>
+        <v>44.04</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>25.72</v>
+        <v>26.56</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>67.8</v>
+        <v>67.94</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.42</v>
+        <v>47.16</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.65</v>
+        <v>29.25</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.78</v>
+        <v>68.91</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>30.09</v>
+        <v>32.04</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.55</v>
+        <v>79.02</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>25.26</v>
+        <v>26.56</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>53.88</v>
+        <v>58.44</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>40.69</v>
+        <v>42.69</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>23.44</v>
+        <v>26.62</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>58.3</v>
+        <v>60.36</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>45.62</v>
+        <v>44.96</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>32.35</v>
+        <v>30.76</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>61.88</v>
+        <v>59.94</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>349008</v>
+        <v>335060</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.57</v>
+        <v>18.79</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1218722</v>
+        <v>1267410</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>68.34</v>
+        <v>71.06999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>215334</v>
+        <v>180651</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>12.08</v>
+        <v>10.13</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>167</v>
+        <v>110</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-15
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-12.tif</t>
+          <t>fli_fars_2026-10-15.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>83.05</v>
+        <v>81.33</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>34.16</v>
+        <v>29.46</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.64</v>
+        <v>43.27</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.06</v>
+        <v>16.12</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>75.14</v>
+        <v>73.7</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45.97</v>
+        <v>40.91</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>23.92</v>
+        <v>19.74</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>77.61</v>
+        <v>74.31</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.57</v>
+        <v>14.03</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>58.88</v>
+        <v>56.91</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44.2</v>
+        <v>39.07</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>29.93</v>
+        <v>24.66</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>69.48</v>
+        <v>64.94</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>42.99</v>
+        <v>35.01</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>27.78</v>
+        <v>17.51</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>62.42</v>
+        <v>58.75</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>54.55</v>
+        <v>41.3</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>33.89</v>
+        <v>20.56</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>74.66</v>
+        <v>61.57</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.93</v>
+        <v>31.6</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>59.93</v>
+        <v>55.25</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>35.27</v>
+        <v>27.26</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>25.04</v>
+        <v>12.57</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>54.93</v>
+        <v>51.07</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>25.27</v>
+        <v>22.68</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>57.01</v>
+        <v>56.9</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>44.46</v>
+        <v>34.53</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.55</v>
+        <v>16</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>63.97</v>
+        <v>58.64</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46.88</v>
+        <v>41.87</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>25.93</v>
+        <v>23.02</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>76.59999999999999</v>
+        <v>69.66</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.42</v>
+        <v>39.42</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>26.95</v>
+        <v>23.01</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>69.41</v>
+        <v>67.86</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.9</v>
+        <v>22.24</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>56.06</v>
+        <v>51.35</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.35</v>
+        <v>22.05</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.32</v>
+        <v>54.35</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>52.22</v>
+        <v>43.47</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>27.99</v>
+        <v>11.14</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>73.47</v>
+        <v>71.25</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.24</v>
+        <v>28.22</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.77</v>
+        <v>57.31</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>31.84</v>
+        <v>19.65</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>56.72</v>
+        <v>44.97</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.22</v>
+        <v>33.95</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>64.18000000000001</v>
+        <v>60.05</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>49.12</v>
+        <v>47</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>32.33</v>
+        <v>27.53</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.59999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>44.01</v>
+        <v>38.52</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>26.18</v>
+        <v>15.55</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>65.14</v>
+        <v>62.54</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>14.25</v>
+        <v>10.38</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>45.57</v>
+        <v>35.73</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.43</v>
+        <v>32.67</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.88</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>63.6</v>
+        <v>57.73</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45.83</v>
+        <v>37.12</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.57</v>
+        <v>17.71</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>71.67</v>
+        <v>63.1</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.26</v>
+        <v>15.75</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>60.21</v>
+        <v>63.29</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>46.06</v>
+        <v>29.48</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>30.74</v>
+        <v>15.07</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>57.16</v>
+        <v>42.41</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.470000000000001</v>
+        <v>7.56</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>58.48</v>
+        <v>51.51</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.98</v>
+        <v>9.74</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>47.65</v>
+        <v>44.68</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>41.74</v>
+        <v>37.82</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>25.39</v>
+        <v>18.85</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>71.75</v>
+        <v>68.23999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>15.54</v>
+        <v>14.23</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>41.27</v>
+        <v>39.7</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>44.04</v>
+        <v>38.55</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>26.56</v>
+        <v>18.7</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>67.94</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>47.16</v>
+        <v>42.58</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>29.25</v>
+        <v>22.76</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>68.91</v>
+        <v>63.5</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.04</v>
+        <v>29.58</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>79.02</v>
+        <v>69.97</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>26.56</v>
+        <v>24.6</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>58.44</v>
+        <v>55.32</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>42.69</v>
+        <v>24.18</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>26.62</v>
+        <v>6.8</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>60.36</v>
+        <v>44.24</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>44.96</v>
+        <v>38.87</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>30.76</v>
+        <v>22.67</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>59.94</v>
+        <v>57.17</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>335060</v>
+        <v>562654</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.79</v>
+        <v>31.55</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1267410</v>
+        <v>1152633</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>71.06999999999999</v>
+        <v>64.64</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>180651</v>
+        <v>67893</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>10.13</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="5">
@@ -1997,10 +1997,10 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>110</v>
+        <v>51</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-16
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-15.tif</t>
+          <t>fli_fars_2026-10-16.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>81.33</v>
+        <v>80.41</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>29.46</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>43.27</v>
+        <v>42.91</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>16.12</v>
+        <v>12.75</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>73.7</v>
+        <v>73.13</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>40.91</v>
+        <v>26.53</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>19.74</v>
+        <v>3.28</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>74.31</v>
+        <v>63.4</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.03</v>
+        <v>16.4</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>56.91</v>
+        <v>64.12</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.07</v>
+        <v>40.24</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>24.66</v>
+        <v>25.79</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>64.94</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>35.01</v>
+        <v>35.14</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>17.51</v>
+        <v>19.14</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>58.75</v>
+        <v>55.05</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>41.3</v>
+        <v>42.07</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>20.56</v>
+        <v>21.6</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>61.57</v>
+        <v>62.37</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>31.6</v>
+        <v>33.42</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.25</v>
+        <v>58.46</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>27.26</v>
+        <v>36.23</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>12.57</v>
+        <v>23.32</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>51.07</v>
+        <v>57.75</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.68</v>
+        <v>22.86</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>56.9</v>
+        <v>53.9</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>34.53</v>
+        <v>38.77</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>16</v>
+        <v>17.63</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>58.64</v>
+        <v>63.49</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>41.87</v>
+        <v>42.14</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>23.02</v>
+        <v>22.43</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.66</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>39.42</v>
+        <v>40.24</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>23.01</v>
+        <v>24.28</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>67.86</v>
+        <v>69.03</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.24</v>
+        <v>22.17</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>51.35</v>
+        <v>52.01</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.05</v>
+        <v>22.42</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>54.35</v>
+        <v>58.48</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>43.47</v>
+        <v>43.53</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>11.14</v>
+        <v>18.88</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>71.25</v>
+        <v>68.23</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.22</v>
+        <v>30.14</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>57.31</v>
+        <v>60.68</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>19.65</v>
+        <v>29.4</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>44.97</v>
+        <v>54.94</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>33.95</v>
+        <v>34.84</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>60.05</v>
+        <v>61.78</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47</v>
+        <v>43.7</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>27.53</v>
+        <v>25.98</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.3</v>
+        <v>62.71</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>38.52</v>
+        <v>39.81</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>15.55</v>
+        <v>19.14</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>62.54</v>
+        <v>62.68</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>10.38</v>
+        <v>12.3</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>35.73</v>
+        <v>37.82</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>32.67</v>
+        <v>36.58</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>8.039999999999999</v>
+        <v>12.55</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>57.73</v>
+        <v>59.4</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>37.12</v>
+        <v>32.46</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>17.71</v>
+        <v>9.42</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>63.1</v>
+        <v>63.71</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.75</v>
+        <v>15.86</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.29</v>
+        <v>63.03</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>29.48</v>
+        <v>30.4</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>15.07</v>
+        <v>13.08</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>42.41</v>
+        <v>42.44</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>7.56</v>
+        <v>8.07</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>51.51</v>
+        <v>50.41</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.74</v>
+        <v>9.15</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>44.68</v>
+        <v>41.74</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>37.82</v>
+        <v>38.76</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>18.85</v>
+        <v>14.89</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>68.23999999999999</v>
+        <v>66.89</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.23</v>
+        <v>16.53</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>39.7</v>
+        <v>43.39</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>38.55</v>
+        <v>33.93</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>18.7</v>
+        <v>10.4</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>64.79000000000001</v>
+        <v>62.6</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.58</v>
+        <v>40.07</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>22.76</v>
+        <v>22.39</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>63.5</v>
+        <v>60</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>29.58</v>
+        <v>28.71</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.97</v>
+        <v>72.98</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.6</v>
+        <v>23.54</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.32</v>
+        <v>51.92</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,20 +1828,20 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>24.18</v>
+        <v>26.17</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>6.8</v>
+        <v>5.53</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>44.24</v>
+        <v>47.44</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>38.87</v>
+        <v>34.32</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>22.67</v>
+        <v>12.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.17</v>
+        <v>56.37</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>562654</v>
+        <v>501514</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>31.55</v>
+        <v>28.12</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1152633</v>
+        <v>1205729</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>64.64</v>
+        <v>67.61</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>67893</v>
+        <v>75947</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3.81</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-17
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-16.tif</t>
+          <t>fli_fars_2026-10-17.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>80.41</v>
+        <v>80.42</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>30.4</v>
+        <v>32.21</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.91</v>
+        <v>45.95</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>12.75</v>
+        <v>22.23</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>73.13</v>
+        <v>73.45</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>26.53</v>
+        <v>38.74</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>3.28</v>
+        <v>16.22</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>63.4</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.4</v>
+        <v>16.59</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>64.12</v>
+        <v>63.01</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>40.24</v>
+        <v>41.39</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>25.79</v>
+        <v>26.78</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>65.90000000000001</v>
+        <v>66.58</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>35.14</v>
+        <v>36.63</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>19.14</v>
+        <v>19.62</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>55.05</v>
+        <v>57.44</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>42.07</v>
+        <v>46.22</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>21.6</v>
+        <v>25.91</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>62.37</v>
+        <v>68.67</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.42</v>
+        <v>34.9</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>58.46</v>
+        <v>60.06</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>36.23</v>
+        <v>34.68</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>23.32</v>
+        <v>22.56</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>57.75</v>
+        <v>54.9</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.86</v>
+        <v>22.25</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>53.9</v>
+        <v>54.7</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>38.77</v>
+        <v>42.47</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>17.63</v>
+        <v>23.69</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>63.49</v>
+        <v>63.82</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>42.14</v>
+        <v>43.25</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>22.43</v>
+        <v>22.44</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>71.40000000000001</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>40.24</v>
+        <v>43.21</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>24.28</v>
+        <v>23.81</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>69.03</v>
+        <v>65.03</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.17</v>
+        <v>22.26</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>52.01</v>
+        <v>55.07</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.42</v>
+        <v>23.14</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.48</v>
+        <v>58.44</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>43.53</v>
+        <v>47.28</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>18.88</v>
+        <v>21.93</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>68.23</v>
+        <v>69.62</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>30.14</v>
+        <v>30.85</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>60.68</v>
+        <v>60.77</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>29.4</v>
+        <v>31.32</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>54.94</v>
+        <v>56.39</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>34.84</v>
+        <v>38.58</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>61.78</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>43.7</v>
+        <v>46.08</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>25.98</v>
+        <v>28.67</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>62.71</v>
+        <v>64.23</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>39.81</v>
+        <v>41.62</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>19.14</v>
+        <v>23.24</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>62.68</v>
+        <v>63.1</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.3</v>
+        <v>12.77</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>37.82</v>
+        <v>38.92</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>36.58</v>
+        <v>38.44</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>12.55</v>
+        <v>18.86</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>59.4</v>
+        <v>59.6</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>32.46</v>
+        <v>37.89</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>9.42</v>
+        <v>20.52</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>63.71</v>
+        <v>64.86</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.86</v>
+        <v>15.74</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.03</v>
+        <v>63.73</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>30.4</v>
+        <v>36.05</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>13.08</v>
+        <v>21.82</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>42.44</v>
+        <v>47.64</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.07</v>
+        <v>8.49</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>50.41</v>
+        <v>49.96</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.15</v>
+        <v>9.52</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>41.74</v>
+        <v>43.16</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.76</v>
+        <v>40.04</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>14.89</v>
+        <v>22.45</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>66.89</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>16.53</v>
+        <v>16.3</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>43.39</v>
+        <v>43.48</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>33.93</v>
+        <v>40.62</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>10.4</v>
+        <v>21.18</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>62.6</v>
+        <v>64.03</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>40.07</v>
+        <v>41.66</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>22.39</v>
+        <v>21.78</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>60</v>
+        <v>62.55</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>28.71</v>
+        <v>29.23</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.98</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>23.54</v>
+        <v>24.54</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>51.92</v>
+        <v>55.31</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>26.17</v>
+        <v>33.25</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>5.53</v>
+        <v>15.08</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>47.44</v>
+        <v>51.36</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>34.32</v>
+        <v>40.58</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>12.45</v>
+        <v>25.93</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.37</v>
+        <v>57.58</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>501514</v>
+        <v>408814</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.12</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1205729</v>
+        <v>1264882</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>67.61</v>
+        <v>70.93000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>75947</v>
+        <v>109499</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>4.26</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-19
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-17.tif</t>
+          <t>fli_fars_2026-10-19.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>80.42</v>
+        <v>80.13</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>32.21</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>45.95</v>
+        <v>44.03</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>22.23</v>
+        <v>19.02</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>73.45</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>38.74</v>
+        <v>41.22</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>16.22</v>
+        <v>20.42</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>68.45999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>16.59</v>
+        <v>10.09</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.01</v>
+        <v>46.86</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.39</v>
+        <v>40.56</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>26.78</v>
+        <v>26.26</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.58</v>
+        <v>66.03</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>36.63</v>
+        <v>38.92</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>19.62</v>
+        <v>22.98</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>57.44</v>
+        <v>59.52</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46.22</v>
+        <v>43.59</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>25.91</v>
+        <v>22.62</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>68.67</v>
+        <v>63.4</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>34.9</v>
+        <v>31.76</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>60.06</v>
+        <v>55.27</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,20 +928,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>34.68</v>
+        <v>15.88</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>22.56</v>
+        <v>4.58</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>54.9</v>
+        <v>35.05</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.25</v>
+        <v>22.84</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>54.7</v>
+        <v>54.73</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.47</v>
+        <v>39.15</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>23.69</v>
+        <v>19.82</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>63.82</v>
+        <v>61.14</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>43.25</v>
+        <v>44.33</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>22.44</v>
+        <v>22.14</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.93000000000001</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>43.21</v>
+        <v>41.89</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>23.81</v>
+        <v>22.2</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>65.03</v>
+        <v>67.44</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.26</v>
+        <v>21.02</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>55.07</v>
+        <v>52.07</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.14</v>
+        <v>23.43</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.44</v>
+        <v>58.46</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>47.28</v>
+        <v>45.67</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>21.93</v>
+        <v>20.48</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>69.62</v>
+        <v>68.97</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>30.85</v>
+        <v>26.55</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>60.77</v>
+        <v>53.5</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>31.32</v>
+        <v>16.18</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>56.39</v>
+        <v>44.77</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>38.58</v>
+        <v>37.63</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>65.09999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46.08</v>
+        <v>44.78</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>28.67</v>
+        <v>25.44</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>64.23</v>
+        <v>63.57</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>41.62</v>
+        <v>39.02</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>23.24</v>
+        <v>20.4</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>63.1</v>
+        <v>60.45</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.77</v>
+        <v>10.86</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>38.92</v>
+        <v>40.45</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>38.44</v>
+        <v>39.04</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>18.86</v>
+        <v>19.44</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>59.6</v>
+        <v>60.74</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>37.89</v>
+        <v>41.45</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>20.52</v>
+        <v>24.87</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>64.86</v>
+        <v>64.84</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.74</v>
+        <v>14.91</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>63.73</v>
+        <v>58.95</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>36.05</v>
+        <v>35.63</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>21.82</v>
+        <v>19.65</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>47.64</v>
+        <v>46.86</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.49</v>
+        <v>7.09</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>49.96</v>
+        <v>45.99</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.52</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>43.16</v>
+        <v>44.61</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>40.04</v>
+        <v>38.32</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>22.45</v>
+        <v>21.16</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>68.45999999999999</v>
+        <v>66.14</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>16.3</v>
+        <v>11.46</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>43.48</v>
+        <v>28.58</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>40.62</v>
+        <v>39.67</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>21.18</v>
+        <v>20.46</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>64.03</v>
+        <v>63.75</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>41.66</v>
+        <v>41.26</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>21.78</v>
+        <v>22.24</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>62.55</v>
+        <v>61.65</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>29.23</v>
+        <v>27.83</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.93000000000001</v>
+        <v>69.53</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.54</v>
+        <v>23.21</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.31</v>
+        <v>52.27</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>33.25</v>
+        <v>34.56</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>15.08</v>
+        <v>16.92</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>51.36</v>
+        <v>50.65</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>40.58</v>
+        <v>42.98</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>25.93</v>
+        <v>28.85</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.58</v>
+        <v>59.64</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>408814</v>
+        <v>531733</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>22.93</v>
+        <v>29.82</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1264882</v>
+        <v>1167075</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>70.93000000000001</v>
+        <v>65.45</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>109499</v>
+        <v>84387</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>6.14</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-20
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-19.tif</t>
+          <t>fli_fars_2026-10-20.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>80.13</v>
+        <v>79.56999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>30.4</v>
+        <v>29.47</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>44.03</v>
+        <v>42.87</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.02</v>
+        <v>17.75</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>72.70999999999999</v>
+        <v>72.20999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.22</v>
+        <v>39.62</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>20.42</v>
+        <v>19.96</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>71.90000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>10.09</v>
+        <v>15.27</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>46.86</v>
+        <v>60.26</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>40.56</v>
+        <v>39.05</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>26.26</v>
+        <v>23.82</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.03</v>
+        <v>63.59</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>38.92</v>
+        <v>36.22</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>22.98</v>
+        <v>20.23</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.52</v>
+        <v>56.33</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>43.59</v>
+        <v>43.7</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>22.62</v>
+        <v>23.67</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>63.4</v>
+        <v>64.45</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>31.76</v>
+        <v>30.1</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.27</v>
+        <v>52.7</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,20 +928,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>15.88</v>
+        <v>32.42</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>4.58</v>
+        <v>22.33</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>35.05</v>
+        <v>53.35</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.84</v>
+        <v>22.23</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>54.73</v>
+        <v>53.82</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>39.15</v>
+        <v>38.14</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>19.82</v>
+        <v>20.31</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.14</v>
+        <v>58.9</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.33</v>
+        <v>41.22</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>22.14</v>
+        <v>22.08</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.18000000000001</v>
+        <v>69.26000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>41.89</v>
+        <v>36.43</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>22.2</v>
+        <v>19.25</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>67.44</v>
+        <v>59.53</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>21.02</v>
+        <v>20.28</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>23.43</v>
+        <v>21.24</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>58.46</v>
+        <v>53.52</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>45.67</v>
+        <v>45.34</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>20.48</v>
+        <v>21.28</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>68.97</v>
+        <v>68.66</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.55</v>
+        <v>26.75</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53.5</v>
+        <v>54.09</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>16.18</v>
+        <v>18.95</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>44.77</v>
+        <v>41.31</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.63</v>
+        <v>33.61</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>64.8</v>
+        <v>59.01</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>44.78</v>
+        <v>44.74</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>25.44</v>
+        <v>26.29</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>63.57</v>
+        <v>63.66</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>39.02</v>
+        <v>38.24</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>20.4</v>
+        <v>19.86</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>60.45</v>
+        <v>59.93</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>10.86</v>
+        <v>12.75</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>40.45</v>
+        <v>40.58</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39.04</v>
+        <v>37.71</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.44</v>
+        <v>19.59</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>60.74</v>
+        <v>58.87</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.45</v>
+        <v>37.14</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>24.87</v>
+        <v>20.18</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>64.84</v>
+        <v>61.25</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.91</v>
+        <v>14.22</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>58.95</v>
+        <v>56.5</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>35.63</v>
+        <v>35.83</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>19.65</v>
+        <v>20.09</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46.86</v>
+        <v>47.05</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>7.09</v>
+        <v>8.27</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>45.99</v>
+        <v>49.88</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>8.710000000000001</v>
+        <v>9.98</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>44.61</v>
+        <v>44.43</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.32</v>
+        <v>38.54</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>21.16</v>
+        <v>20.74</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>66.14</v>
+        <v>67.58</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>11.46</v>
+        <v>14.67</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>28.58</v>
+        <v>40.87</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>39.67</v>
+        <v>39.08</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>20.46</v>
+        <v>21.48</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>63.75</v>
+        <v>63.28</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>41.26</v>
+        <v>39.72</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>22.24</v>
+        <v>21.68</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.65</v>
+        <v>60.44</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>27.83</v>
+        <v>28.39</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.53</v>
+        <v>69.52</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>23.21</v>
+        <v>23.35</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>52.27</v>
+        <v>51.63</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>34.56</v>
+        <v>33.29</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>16.92</v>
+        <v>15.18</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>50.65</v>
+        <v>50.47</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>42.98</v>
+        <v>40.67</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>28.85</v>
+        <v>26.5</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>59.64</v>
+        <v>57.18</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>531733</v>
+        <v>553180</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>29.82</v>
+        <v>31.02</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1167075</v>
+        <v>1172193</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>65.45</v>
+        <v>65.73</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>84387</v>
+        <v>57833</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>4.73</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-21
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-20.tif</t>
+          <t>fli_fars_2026-10-21.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>79.56999999999999</v>
+        <v>78.7</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>29.47</v>
+        <v>29.89</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.87</v>
+        <v>43.53</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.75</v>
+        <v>19.32</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>72.20999999999999</v>
+        <v>71.65000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>39.62</v>
+        <v>38.71</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>19.96</v>
+        <v>19.76</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>71.2</v>
+        <v>70.56</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.27</v>
+        <v>15.75</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>60.26</v>
+        <v>61.4</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.05</v>
+        <v>41.07</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>23.82</v>
+        <v>26.31</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>63.59</v>
+        <v>66.73</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>36.22</v>
+        <v>38.35</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>20.23</v>
+        <v>21.93</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>56.33</v>
+        <v>59.15</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -867,10 +867,10 @@
         <v>43.7</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>23.67</v>
+        <v>23.6</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>64.45</v>
+        <v>64.78</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>30.1</v>
+        <v>29.85</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>52.7</v>
+        <v>52.79</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>32.42</v>
+        <v>31.87</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>22.33</v>
+        <v>21.8</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>53.35</v>
+        <v>52.4</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.23</v>
+        <v>22.41</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>53.82</v>
+        <v>54.09</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>38.14</v>
+        <v>37.8</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>20.31</v>
+        <v>21.04</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>58.9</v>
+        <v>57.78</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>41.22</v>
+        <v>40.41</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>22.08</v>
+        <v>21.07</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.26000000000001</v>
+        <v>68.94</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>36.43</v>
+        <v>36.54</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>19.25</v>
+        <v>15.95</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>59.53</v>
+        <v>64.91</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.28</v>
+        <v>20.66</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.54</v>
+        <v>48.88</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.24</v>
+        <v>21.39</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>53.52</v>
+        <v>53.74</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>45.34</v>
+        <v>46.27</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>21.28</v>
+        <v>21.04</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>68.66</v>
+        <v>68.95</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.75</v>
+        <v>25.15</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>54.09</v>
+        <v>50.94</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>18.95</v>
+        <v>25.01</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>41.31</v>
+        <v>46.11</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>33.61</v>
+        <v>31.74</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>59.01</v>
+        <v>57.7</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>44.74</v>
+        <v>45.09</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>26.29</v>
+        <v>25.83</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>63.66</v>
+        <v>64.47</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>38.24</v>
+        <v>37.93</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>19.86</v>
+        <v>20.59</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>59.93</v>
+        <v>60.99</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.75</v>
+        <v>13.4</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>40.58</v>
+        <v>43.93</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>37.71</v>
+        <v>37.69</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.59</v>
+        <v>17.55</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>58.87</v>
+        <v>59.07</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>37.14</v>
+        <v>37.59</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>20.18</v>
+        <v>22.08</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>61.25</v>
+        <v>63.65</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.22</v>
+        <v>15.14</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>56.5</v>
+        <v>60.09</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>35.83</v>
+        <v>34.99</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>20.09</v>
+        <v>19.91</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>47.05</v>
+        <v>46.02</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.27</v>
+        <v>8.67</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.98</v>
+        <v>10.06</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>44.43</v>
+        <v>44.08</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.54</v>
+        <v>38.55</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>20.74</v>
+        <v>21.25</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>67.58</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.67</v>
+        <v>15.59</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>40.87</v>
+        <v>41.51</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>39.08</v>
+        <v>37.05</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>21.48</v>
+        <v>16.76</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>63.28</v>
+        <v>62.11</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>39.72</v>
+        <v>41.38</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>21.68</v>
+        <v>22.96</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>60.44</v>
+        <v>62.66</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>28.39</v>
+        <v>29.76</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.52</v>
+        <v>71.41</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>23.35</v>
+        <v>24.51</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>51.63</v>
+        <v>55.53</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>33.29</v>
+        <v>31.8</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>15.18</v>
+        <v>14.32</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>50.47</v>
+        <v>48.05</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>40.67</v>
+        <v>40.51</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>26.5</v>
+        <v>26.42</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.18</v>
+        <v>56.89</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>553180</v>
+        <v>513240</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>31.02</v>
+        <v>28.78</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1172193</v>
+        <v>1208485</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>65.73</v>
+        <v>67.77</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>57833</v>
+        <v>61479</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3.24</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-22
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-21.tif</t>
+          <t>fli_fars_2026-10-22.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>78.7</v>
+        <v>82.67</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>29.89</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>43.53</v>
+        <v>46.48</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.32</v>
+        <v>22.86</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>71.65000000000001</v>
+        <v>74.13</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>38.71</v>
+        <v>41.89</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>19.76</v>
+        <v>21.08</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>70.56</v>
+        <v>72.67</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.75</v>
+        <v>14.49</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>61.4</v>
+        <v>54.93</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.07</v>
+        <v>38.36</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>26.31</v>
+        <v>23.92</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.73</v>
+        <v>63.91</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>38.35</v>
+        <v>38.48</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>21.93</v>
+        <v>23.12</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.15</v>
+        <v>59.04</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>43.7</v>
+        <v>50.34</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>23.6</v>
+        <v>30.09</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>64.78</v>
+        <v>72.26000000000001</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>29.85</v>
+        <v>30.25</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>52.79</v>
+        <v>53.01</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>31.87</v>
+        <v>29.46</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>21.8</v>
+        <v>18.69</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>52.4</v>
+        <v>49.51</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.41</v>
+        <v>22.74</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>54.09</v>
+        <v>53.8</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>37.8</v>
+        <v>42.16</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>21.04</v>
+        <v>24.55</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>57.78</v>
+        <v>61.91</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>40.41</v>
+        <v>43.03</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>21.07</v>
+        <v>23</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>68.94</v>
+        <v>72.51000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>36.54</v>
+        <v>40.65</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>15.95</v>
+        <v>20.65</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>64.91</v>
+        <v>65.88</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.66</v>
+        <v>20.95</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.88</v>
+        <v>51.7</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.39</v>
+        <v>22.34</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>53.74</v>
+        <v>54.03</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46.27</v>
+        <v>49.36</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>21.04</v>
+        <v>24.51</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>68.95</v>
+        <v>70.54000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>25.15</v>
+        <v>25.66</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>50.94</v>
+        <v>52.58</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>25.01</v>
+        <v>27.07</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>46.11</v>
+        <v>48.69</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>31.74</v>
+        <v>34.07</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>57.7</v>
+        <v>59.5</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>45.09</v>
+        <v>48.53</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>25.83</v>
+        <v>31.22</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>64.47</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>37.93</v>
+        <v>41.93</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>20.59</v>
+        <v>24.67</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>60.99</v>
+        <v>61.55</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.4</v>
+        <v>12.95</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>43.93</v>
+        <v>41.05</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>37.69</v>
+        <v>42.72</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>17.55</v>
+        <v>21.51</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>59.07</v>
+        <v>63.19</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>37.59</v>
+        <v>40.3</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>22.08</v>
+        <v>22.77</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>63.65</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.14</v>
+        <v>15.04</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>60.09</v>
+        <v>61.49</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>34.99</v>
+        <v>44.13</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>19.91</v>
+        <v>28.95</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46.02</v>
+        <v>55.18</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.67</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>49.88</v>
+        <v>48.76</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>10.06</v>
+        <v>9.44</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>44.08</v>
+        <v>43.77</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.55</v>
+        <v>39.7</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>21.25</v>
+        <v>23.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>67.40000000000001</v>
+        <v>66.58</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>15.59</v>
+        <v>14.25</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>41.51</v>
+        <v>35.41</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>37.05</v>
+        <v>42.14</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>16.76</v>
+        <v>24.78</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>62.11</v>
+        <v>63.69</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>41.38</v>
+        <v>44.5</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>22.96</v>
+        <v>25.8</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>62.66</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>29.76</v>
+        <v>29.33</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>71.41</v>
+        <v>72.27</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.51</v>
+        <v>24.68</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.53</v>
+        <v>54.4</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>31.8</v>
+        <v>38.72</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>14.32</v>
+        <v>21.87</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.05</v>
+        <v>55.61</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>40.51</v>
+        <v>47.12</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>26.42</v>
+        <v>33.58</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.89</v>
+        <v>62.75</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>513240</v>
+        <v>426287</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.78</v>
+        <v>23.91</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1208485</v>
+        <v>1260822</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>67.77</v>
+        <v>70.7</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>61479</v>
+        <v>96034</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3.45</v>
+        <v>5.39</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-23
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-22.tif</t>
+          <t>fli_fars_2026-10-23.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>82.67</v>
+        <v>80.88</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>31.4</v>
+        <v>29.85</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46.48</v>
+        <v>40.73</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>22.86</v>
+        <v>11.49</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>74.13</v>
+        <v>69.23</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.89</v>
+        <v>41.83</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>21.08</v>
+        <v>21.99</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>72.67</v>
+        <v>73.72</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.49</v>
+        <v>11.05</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>54.93</v>
+        <v>43.85</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>38.36</v>
+        <v>36.79</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>23.92</v>
+        <v>21.65</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>63.91</v>
+        <v>61.5</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>38.48</v>
+        <v>37</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>23.12</v>
+        <v>21.53</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.04</v>
+        <v>57.3</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>50.34</v>
+        <v>51.29</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>30.09</v>
+        <v>29.51</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>72.26000000000001</v>
+        <v>71.34999999999999</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>30.25</v>
+        <v>33.42</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>53.01</v>
+        <v>58.24</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>29.46</v>
+        <v>27.44</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>18.69</v>
+        <v>16.17</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>49.51</v>
+        <v>50.04</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.74</v>
+        <v>22.86</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>53.8</v>
+        <v>52.74</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.16</v>
+        <v>37.42</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>24.55</v>
+        <v>20.19</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.91</v>
+        <v>58.29</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>43.03</v>
+        <v>41.71</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>23</v>
+        <v>22.27</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.51000000000001</v>
+        <v>70.03</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>40.65</v>
+        <v>39.15</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>20.65</v>
+        <v>19.16</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>65.88</v>
+        <v>63.05</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.95</v>
+        <v>20.92</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>51.7</v>
+        <v>52.33</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.34</v>
+        <v>22.1</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>54.03</v>
+        <v>56.48</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>49.36</v>
+        <v>46.4</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>24.51</v>
+        <v>20.98</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>70.54000000000001</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>25.66</v>
+        <v>27.94</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>52.58</v>
+        <v>56.75</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>27.07</v>
+        <v>20.35</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>48.69</v>
+        <v>44</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>34.07</v>
+        <v>36.4</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>59.5</v>
+        <v>62.57</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>48.53</v>
+        <v>43.72</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>31.22</v>
+        <v>26.18</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>67.18000000000001</v>
+        <v>61.74</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>41.93</v>
+        <v>38.31</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>24.67</v>
+        <v>19.73</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>61.55</v>
+        <v>58.83</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.95</v>
+        <v>10.16</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>41.05</v>
+        <v>31.9</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>42.72</v>
+        <v>32.47</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>21.51</v>
+        <v>12.86</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>63.19</v>
+        <v>54.47</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>40.3</v>
+        <v>40.02</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>22.77</v>
+        <v>23.12</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>64.73999999999999</v>
+        <v>64.51000000000001</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.04</v>
+        <v>15.4</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>61.49</v>
+        <v>62.84</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44.13</v>
+        <v>34.68</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>28.95</v>
+        <v>19.85</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>55.18</v>
+        <v>45.67</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.369999999999999</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>48.76</v>
+        <v>48.57</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.44</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>43.77</v>
+        <v>42.34</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>39.7</v>
+        <v>38.56</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>23.01</v>
+        <v>18.8</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>66.58</v>
+        <v>70.03</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.25</v>
+        <v>12.79</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>35.41</v>
+        <v>33.43</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>42.14</v>
+        <v>42.35</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>24.78</v>
+        <v>24.6</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>63.69</v>
+        <v>64.81</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>44.5</v>
+        <v>39.58</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.8</v>
+        <v>21.12</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>66.29000000000001</v>
+        <v>59.81</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>29.33</v>
+        <v>27.5</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>72.27</v>
+        <v>73.61</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>24.68</v>
+        <v>22.84</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>54.4</v>
+        <v>53.99</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>38.72</v>
+        <v>31.74</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>21.87</v>
+        <v>15.49</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>55.61</v>
+        <v>49.84</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>47.12</v>
+        <v>43.6</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>33.58</v>
+        <v>29.81</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.75</v>
+        <v>59.78</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>426287</v>
+        <v>543186</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>23.91</v>
+        <v>30.46</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1260822</v>
+        <v>1170323</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>70.7</v>
+        <v>65.63</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>96034</v>
+        <v>69697</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>5.39</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-25
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-23.tif</t>
+          <t>fli_fars_2026-10-25.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>80.88</v>
+        <v>84.81999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>29.85</v>
+        <v>31.87</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>40.73</v>
+        <v>44.27</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>11.49</v>
+        <v>20.86</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>69.23</v>
+        <v>71.75</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.83</v>
+        <v>43.66</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>21.99</v>
+        <v>22.41</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>73.72</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>11.05</v>
+        <v>14.64</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>43.85</v>
+        <v>57.9</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>36.79</v>
+        <v>39.93</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>21.65</v>
+        <v>25.12</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>61.5</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>37</v>
+        <v>38.56</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>21.53</v>
+        <v>18.29</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>57.3</v>
+        <v>60.65</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.29</v>
+        <v>55.82</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>29.51</v>
+        <v>32.21</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>71.34999999999999</v>
+        <v>76.16</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.42</v>
+        <v>36.45</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>58.24</v>
+        <v>62.62</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>27.44</v>
+        <v>29.41</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>16.17</v>
+        <v>18.57</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>50.04</v>
+        <v>50.59</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>22.86</v>
+        <v>24.31</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>52.74</v>
+        <v>54.93</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>37.42</v>
+        <v>40.8</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>20.19</v>
+        <v>17.77</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>58.29</v>
+        <v>64.95999999999999</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>41.71</v>
+        <v>42.08</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>22.27</v>
+        <v>21.04</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>70.03</v>
+        <v>70.63</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>39.15</v>
+        <v>38.23</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>19.16</v>
+        <v>20.16</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>63.05</v>
+        <v>62.79</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.92</v>
+        <v>20.47</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>52.33</v>
+        <v>48.23</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.1</v>
+        <v>22.08</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.48</v>
+        <v>56.18</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46.4</v>
+        <v>50.1</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>20.98</v>
+        <v>25.14</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>68.84999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>خیلی زیاد</t>
         </is>
       </c>
     </row>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.94</v>
+        <v>31.11</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>56.75</v>
+        <v>59.76</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>20.35</v>
+        <v>24.94</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>44</v>
+        <v>47.77</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>36.4</v>
+        <v>37.14</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>62.57</v>
+        <v>63.31</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>43.72</v>
+        <v>47.38</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>26.18</v>
+        <v>29.13</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>61.74</v>
+        <v>66.48</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>38.31</v>
+        <v>40.73</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>19.73</v>
+        <v>23.76</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>58.83</v>
+        <v>60.94</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>10.16</v>
+        <v>12.5</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>31.9</v>
+        <v>37.83</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>32.47</v>
+        <v>30.96</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>12.86</v>
+        <v>6.12</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>54.47</v>
+        <v>54.08</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>40.02</v>
+        <v>39.37</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>23.12</v>
+        <v>22.11</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>64.51000000000001</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.4</v>
+        <v>14.49</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>62.84</v>
+        <v>57.01</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>34.68</v>
+        <v>45.08</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>19.85</v>
+        <v>28.18</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>45.67</v>
+        <v>56.57</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>8.029999999999999</v>
+        <v>9.58</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>48.57</v>
+        <v>54.56</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>9.119999999999999</v>
+        <v>11.52</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>42.34</v>
+        <v>50.95</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.56</v>
+        <v>39.91</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>18.8</v>
+        <v>23.15</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>70.03</v>
+        <v>68.22</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>12.79</v>
+        <v>14.52</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>33.43</v>
+        <v>39.48</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>42.35</v>
+        <v>40.24</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>24.6</v>
+        <v>23.06</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>64.81</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>39.58</v>
+        <v>45.44</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>21.12</v>
+        <v>25.01</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>59.81</v>
+        <v>65.77</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>27.5</v>
+        <v>32.91</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>73.61</v>
+        <v>74.97</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>22.84</v>
+        <v>28.42</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>53.99</v>
+        <v>59.86</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>31.74</v>
+        <v>30.05</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>15.49</v>
+        <v>9.41</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>49.84</v>
+        <v>53.53</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>43.6</v>
+        <v>44.15</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>29.81</v>
+        <v>28.75</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>59.78</v>
+        <v>59.99</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>543186</v>
+        <v>453368</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>30.46</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1170323</v>
+        <v>1216697</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>65.63</v>
+        <v>68.23</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>69697</v>
+        <v>113134</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3.91</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-26
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-25.tif</t>
+          <t>fli_fars_2026-10-26.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>84.81999999999999</v>
+        <v>84.97</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>31.87</v>
+        <v>32.48</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>44.27</v>
+        <v>44.51</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>20.86</v>
+        <v>19.82</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>71.75</v>
+        <v>73.34999999999999</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.66</v>
+        <v>44.1</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>22.41</v>
+        <v>23.05</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>74.79000000000001</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.64</v>
+        <v>15.29</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>57.9</v>
+        <v>60.5</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.93</v>
+        <v>41.5</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>25.12</v>
+        <v>27.17</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.43000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>38.56</v>
+        <v>39.25</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>18.29</v>
+        <v>22.52</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>60.65</v>
+        <v>59.97</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>55.82</v>
+        <v>53.11</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>32.21</v>
+        <v>28.82</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>76.16</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>36.45</v>
+        <v>33.96</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>62.62</v>
+        <v>59.54</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>29.41</v>
+        <v>30.15</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>18.57</v>
+        <v>19.77</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>50.59</v>
+        <v>49.39</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>24.31</v>
+        <v>25.33</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>54.93</v>
+        <v>56.54</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>40.8</v>
+        <v>36.2</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>17.77</v>
+        <v>19.06</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>64.95999999999999</v>
+        <v>59.25</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>42.08</v>
+        <v>41.29</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>21.04</v>
+        <v>20.18</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>70.63</v>
+        <v>69.63</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>38.23</v>
+        <v>37.57</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>20.16</v>
+        <v>20.71</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>62.79</v>
+        <v>63.98</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.47</v>
+        <v>19.82</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.23</v>
+        <v>50.73</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>22.08</v>
+        <v>21.04</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>56.18</v>
+        <v>54.01</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,20 +1152,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>50.1</v>
+        <v>47.77</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>25.14</v>
+        <v>22.07</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>71.7</v>
+        <v>69.62</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>31.11</v>
+        <v>30.95</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>59.76</v>
+        <v>59.33</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>24.94</v>
+        <v>31.42</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>47.77</v>
+        <v>56.05</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.14</v>
+        <v>37.43</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>63.31</v>
+        <v>63.72</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>47.38</v>
+        <v>46.8</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>29.13</v>
+        <v>28.41</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>66.48</v>
+        <v>65.97</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>40.73</v>
+        <v>37.44</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>23.76</v>
+        <v>19.86</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>60.94</v>
+        <v>58.51</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.5</v>
+        <v>13.12</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>37.83</v>
+        <v>40.32</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>30.96</v>
+        <v>37.53</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>6.12</v>
+        <v>19.24</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>54.08</v>
+        <v>58.94</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>39.37</v>
+        <v>42.04</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>22.11</v>
+        <v>25.78</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.26000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.49</v>
+        <v>14.36</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>57.01</v>
+        <v>57.53</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>45.08</v>
+        <v>43.89</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>28.18</v>
+        <v>25.98</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>56.57</v>
+        <v>55.53</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.58</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.56</v>
+        <v>54.24</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.52</v>
+        <v>11.32</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>50.95</v>
+        <v>49.33</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>39.91</v>
+        <v>40.49</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>23.15</v>
+        <v>23.62</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>68.22</v>
+        <v>70.69</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.52</v>
+        <v>14.69</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>39.48</v>
+        <v>39.51</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>40.24</v>
+        <v>40.3</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>23.06</v>
+        <v>23.3</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>64.04000000000001</v>
+        <v>62.17</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.44</v>
+        <v>48.18</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>25.01</v>
+        <v>27.65</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>65.77</v>
+        <v>69.84</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.91</v>
+        <v>32.37</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>74.97</v>
+        <v>76.45</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>28.42</v>
+        <v>27.7</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>59.86</v>
+        <v>58.26</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>30.05</v>
+        <v>37.02</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>9.41</v>
+        <v>19.41</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>53.53</v>
+        <v>54</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>44.15</v>
+        <v>47.83</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>28.75</v>
+        <v>33.19</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>59.99</v>
+        <v>62.37</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>453368</v>
+        <v>402927</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>25.42</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1216697</v>
+        <v>1258920</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>68.23</v>
+        <v>70.59999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>113134</v>
+        <v>121348</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>6.34</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-28
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-26.tif</t>
+          <t>fli_fars_2026-10-28.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>84.97</v>
+        <v>77.94</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>32.48</v>
+        <v>27.57</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>44.51</v>
+        <v>40.46</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.82</v>
+        <v>11.14</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>73.34999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>44.1</v>
+        <v>37.55</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>23.05</v>
+        <v>17.28</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>74.98999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>15.29</v>
+        <v>14.71</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>60.5</v>
+        <v>58.21</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.5</v>
+        <v>39.06</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>27.17</v>
+        <v>24.45</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>66.8</v>
+        <v>64.72</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>39.25</v>
+        <v>34.59</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>22.52</v>
+        <v>19.22</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>59.97</v>
+        <v>54.91</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,20 +864,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>53.11</v>
+        <v>41.79</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>28.82</v>
+        <v>21.52</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>73.51000000000001</v>
+        <v>62.29</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>خیلی زیاد</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.96</v>
+        <v>30.16</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>59.54</v>
+        <v>53.35</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>30.15</v>
+        <v>32.44</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>19.77</v>
+        <v>23.07</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>49.39</v>
+        <v>53.44</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,20 +960,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>25.33</v>
+        <v>20.31</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>56.54</v>
+        <v>50.59</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>36.2</v>
+        <v>34.42</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>19.06</v>
+        <v>17.49</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>59.25</v>
+        <v>53.86</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>41.29</v>
+        <v>38.79</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>20.18</v>
+        <v>20.11</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>69.63</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>37.57</v>
+        <v>31.08</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>20.71</v>
+        <v>12.93</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>63.98</v>
+        <v>53.8</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>19.82</v>
+        <v>16.76</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>50.73</v>
+        <v>41.33</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>21.04</v>
+        <v>19.19</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>54.01</v>
+        <v>47.64</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>47.77</v>
+        <v>44.47</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>22.07</v>
+        <v>19.23</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>69.62</v>
+        <v>65.73</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>30.95</v>
+        <v>27.01</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>59.33</v>
+        <v>53.9</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,13 +1216,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>31.42</v>
+        <v>25.62</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>56.05</v>
+        <v>51.32</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>37.43</v>
+        <v>30.76</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>63.72</v>
+        <v>56.56</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46.8</v>
+        <v>44.42</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>28.41</v>
+        <v>26.76</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>65.97</v>
+        <v>63.72</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>37.44</v>
+        <v>37.08</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>19.86</v>
+        <v>18.82</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>58.51</v>
+        <v>60.57</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>13.12</v>
+        <v>12.51</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>40.32</v>
+        <v>38.19</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>37.53</v>
+        <v>33.41</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>19.24</v>
+        <v>15.42</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>58.94</v>
+        <v>55.06</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>42.04</v>
+        <v>35.05</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>25.78</v>
+        <v>19.93</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>67.09999999999999</v>
+        <v>59.93</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.36</v>
+        <v>12.93</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>57.53</v>
+        <v>52.37</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>43.89</v>
+        <v>29.32</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>25.98</v>
+        <v>11.73</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>55.53</v>
+        <v>41.01</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.300000000000001</v>
+        <v>7.87</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.24</v>
+        <v>48.06</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>11.32</v>
+        <v>8.82</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>49.33</v>
+        <v>40.85</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>40.49</v>
+        <v>36.08</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>23.62</v>
+        <v>17.05</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>70.69</v>
+        <v>65.56999999999999</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.69</v>
+        <v>14.79</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>39.51</v>
+        <v>37.27</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>40.3</v>
+        <v>35.69</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>23.3</v>
+        <v>16.62</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>62.17</v>
+        <v>60.26</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>48.18</v>
+        <v>37.19</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.65</v>
+        <v>18.18</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>69.84</v>
+        <v>58.81</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>32.37</v>
+        <v>26.41</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>76.45</v>
+        <v>67.63</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,20 +1796,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>27.7</v>
+        <v>21.31</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>58.26</v>
+        <v>51.08</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>37.02</v>
+        <v>28.42</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>19.41</v>
+        <v>9.48</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>54</v>
+        <v>44.89</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>47.83</v>
+        <v>36.45</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>33.19</v>
+        <v>22.02</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.37</v>
+        <v>52.12</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>402927</v>
+        <v>671420</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>22.6</v>
+        <v>37.65</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1258920</v>
+        <v>1078440</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>70.59999999999999</v>
+        <v>60.48</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>121348</v>
+        <v>33357</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>6.8</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-10-29
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-10-28.tif</t>
+          <t>fli_fars_2026-10-29.tif</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>77.94</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="9">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>27.57</v>
+        <v>28.37</v>
       </c>
     </row>
     <row r="10">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>40.46</v>
+        <v>40.19</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>11.14</v>
+        <v>11.22</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>70.40000000000001</v>
+        <v>70.95</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24931</v>
@@ -736,13 +736,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>37.55</v>
+        <v>40.04</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>17.28</v>
+        <v>19.79</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>70.40000000000001</v>
+        <v>70.83</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7596</v>
@@ -768,13 +768,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>14.71</v>
+        <v>13.04</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>58.21</v>
+        <v>52.48</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>14316</v>
@@ -800,13 +800,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.06</v>
+        <v>40.63</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>24.45</v>
+        <v>26.71</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>64.72</v>
+        <v>65.53</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>13047</v>
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>34.59</v>
+        <v>35.57</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>19.22</v>
+        <v>19.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>54.91</v>
+        <v>56.84</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>4435</v>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>41.79</v>
+        <v>46.58</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>21.52</v>
+        <v>25.48</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>62.29</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2330</v>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>30.16</v>
+        <v>30.54</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.43</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>53.35</v>
+        <v>53.09</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4168</v>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>32.44</v>
+        <v>27.92</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>23.07</v>
+        <v>16.7</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>53.44</v>
+        <v>46.73</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1294</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>20.31</v>
+        <v>20.41</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>50.59</v>
+        <v>51.35</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>3417</v>
@@ -992,13 +992,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>34.42</v>
+        <v>34.32</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>17.49</v>
+        <v>12.03</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>53.86</v>
+        <v>59.17</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>4643</v>
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>38.79</v>
+        <v>41.82</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>20.11</v>
+        <v>21</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>67.65000000000001</v>
+        <v>71.08</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>8020</v>
@@ -1056,13 +1056,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>31.08</v>
+        <v>33.59</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>12.93</v>
+        <v>11.73</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>53.8</v>
+        <v>58.26</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>13859</v>
@@ -1088,13 +1088,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>16.76</v>
+        <v>18.43</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0.34</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>41.33</v>
+        <v>43.44</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>10541</v>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>19.19</v>
+        <v>20.54</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.37</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>47.64</v>
+        <v>51.67</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>13329</v>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>44.47</v>
+        <v>42.46</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>19.23</v>
+        <v>18.31</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>65.73</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4909</v>
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.01</v>
+        <v>25.77</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0.73</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>53.9</v>
+        <v>52.8</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>19003</v>
@@ -1216,20 +1216,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>25.62</v>
+        <v>23.7</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.78</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>51.32</v>
+        <v>44.24</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>11473</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>30.76</v>
+        <v>31.96</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>56.56</v>
+        <v>57.86</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>9100</v>
@@ -1280,13 +1280,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>44.42</v>
+        <v>47.36</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>26.76</v>
+        <v>29.82</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>63.72</v>
+        <v>65.86</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>791</v>
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>37.08</v>
+        <v>34.93</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>18.82</v>
+        <v>16.1</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>60.57</v>
+        <v>60.02</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>7038</v>
@@ -1344,13 +1344,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>12.51</v>
+        <v>13.92</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0.51</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>38.19</v>
+        <v>43.09</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>4821</v>
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>33.41</v>
+        <v>38.05</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>15.42</v>
+        <v>16.06</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>55.06</v>
+        <v>60.04</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2287</v>
@@ -1476,13 +1476,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>35.05</v>
+        <v>33.73</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>19.93</v>
+        <v>18.26</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>59.93</v>
+        <v>58.97</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>7892</v>
@@ -1508,13 +1508,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>12.93</v>
+        <v>13.73</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.23</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>52.37</v>
+        <v>54.77</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>18742</v>
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>29.32</v>
+        <v>40.45</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>11.73</v>
+        <v>24.26</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>41.01</v>
+        <v>51.62</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>470</v>
@@ -1572,13 +1572,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>7.87</v>
+        <v>7.75</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0.21</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>48.06</v>
+        <v>47.13</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>43913</v>
@@ -1604,13 +1604,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>8.82</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>0.4</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>40.85</v>
+        <v>41.67</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>4718</v>
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>36.08</v>
+        <v>36.01</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>17.05</v>
+        <v>19.64</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>65.56999999999999</v>
+        <v>65.56</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>8411</v>
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>14.79</v>
+        <v>13.52</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>37.27</v>
+        <v>34.96</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>2525</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>35.69</v>
+        <v>37.42</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>16.62</v>
+        <v>15.35</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>60.26</v>
+        <v>60.86</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>7186</v>
@@ -1732,13 +1732,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>37.19</v>
+        <v>35.94</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>18.18</v>
+        <v>11.33</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>58.81</v>
+        <v>62.42</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>6990</v>
@@ -1764,13 +1764,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>26.41</v>
+        <v>27.36</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>67.63</v>
+        <v>67.38</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>45935</v>
@@ -1796,13 +1796,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>21.31</v>
+        <v>22.78</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>51.08</v>
+        <v>53.31</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>24115</v>
@@ -1828,13 +1828,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>28.42</v>
+        <v>31.86</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>9.48</v>
+        <v>12.98</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>44.89</v>
+        <v>50.33</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2712</v>
@@ -1860,13 +1860,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>36.45</v>
+        <v>38.7</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>22.02</v>
+        <v>20.09</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>52.12</v>
+        <v>51.69</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1692</v>
@@ -1940,10 +1940,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>671420</v>
+        <v>644845</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>37.65</v>
+        <v>36.16</v>
       </c>
     </row>
     <row r="3">
@@ -1959,10 +1959,10 @@
         <v>50</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1078440</v>
+        <v>1091331</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>60.48</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="4">
@@ -1978,10 +1978,10 @@
         <v>75</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>33357</v>
+        <v>46995</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1.87</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="5">
@@ -1997,7 +1997,7 @@
         <v>100</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>

</xml_diff>